<commit_message>
fix(bom-template): purge leftover SimSun font, landscape fit-to-width, full-column print area
- Normalize every rendered cell to Arial (purge 358 leftover 宋/SimSun cells in
  cols P-S and header shadow cells). ZTool's exporter clones the template data
  row's cell style when inserting rows, so any stray SimSun cell made exported
  data render in Chinese font.
- Page setup: landscape, fit-to-width=1, print area A1:O75 (vendor template
  printed only A1:K40, cutting off columns L-O), repeat title+header rows.
- Add reproducible tooling: client-core/tools/fix_template_format.py (path-robust)
  and client-core/tools/make_bom_preview.py (fills template with sample Russian
  data to review formatting without ZTool/SolidWorks).
</commit_message>
<xml_diff>
--- a/Шаблоны спецификации/bom_шаблон.xlsx
+++ b/Шаблоны спецификации/bom_шаблон.xlsx
@@ -26,7 +26,7 @@
     <definedName name="Эскиз">Спецификация!$M$6</definedName>
     <definedName name="Количество">Спецификация!$G$6</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Спецификация'!$1:$6</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Спецификация'!$A$1:$K$40</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Спецификация'!$A$1:$O$75</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -37,7 +37,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0_);[Red]\(0\)"/>
   </numFmts>
-  <fonts count="30">
+  <fonts count="31">
     <font>
       <name val="宋体"/>
       <charset val="134"/>
@@ -239,6 +239,10 @@
       <name val="Arial"/>
       <b val="1"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="12"/>
     </font>
   </fonts>
   <fills count="10">
@@ -585,7 +589,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="56">
+  <cellXfs count="66">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
@@ -734,6 +738,34 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="21" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="22" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="23" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="28" fillId="0" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="28" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="30" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="18">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -1151,7 +1183,7 @@
   <sheetPr codeName="Sheet1">
     <tabColor indexed="53"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:S75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="20.1" customHeight="1"/>
@@ -1179,122 +1211,152 @@
           <t>Спецификация</t>
         </is>
       </c>
+      <c r="B1" s="37" t="n"/>
+      <c r="C1" s="37" t="n"/>
+      <c r="D1" s="37" t="n"/>
+      <c r="E1" s="37" t="n"/>
+      <c r="F1" s="37" t="n"/>
+      <c r="G1" s="37" t="n"/>
+      <c r="H1" s="37" t="n"/>
+      <c r="I1" s="37" t="n"/>
+      <c r="J1" s="37" t="n"/>
+      <c r="K1" s="37" t="n"/>
       <c r="L1" s="37" t="n"/>
       <c r="M1" s="37" t="n"/>
       <c r="N1" s="37" t="n"/>
       <c r="O1" s="37" t="n"/>
+      <c r="P1" s="56" t="n"/>
+      <c r="Q1" s="56" t="n"/>
+      <c r="R1" s="56" t="n"/>
+      <c r="S1" s="56" t="n"/>
     </row>
     <row r="2" ht="16" customHeight="1">
-      <c r="A2" s="38" t="inlineStr">
+      <c r="A2" s="57" t="inlineStr">
         <is>
           <t>Наименование изделия: XXX</t>
         </is>
       </c>
-      <c r="B2" s="34" t="n"/>
-      <c r="C2" s="34" t="n"/>
-      <c r="D2" s="39" t="inlineStr">
+      <c r="B2" s="58" t="n"/>
+      <c r="C2" s="58" t="n"/>
+      <c r="D2" s="58" t="inlineStr">
         <is>
           <t>Обозначение изделия: XXX</t>
         </is>
       </c>
-      <c r="E2" s="34" t="n"/>
-      <c r="F2" s="34" t="n"/>
-      <c r="G2" s="34" t="n"/>
-      <c r="H2" s="34" t="n"/>
-      <c r="I2" s="39" t="inlineStr">
+      <c r="E2" s="58" t="n"/>
+      <c r="F2" s="58" t="n"/>
+      <c r="G2" s="58" t="n"/>
+      <c r="H2" s="58" t="n"/>
+      <c r="I2" s="58" t="inlineStr">
         <is>
           <t>Составил:</t>
         </is>
       </c>
-      <c r="J2" s="39" t="inlineStr">
+      <c r="J2" s="58" t="inlineStr">
         <is>
           <t>Дата:</t>
         </is>
       </c>
-      <c r="K2" s="34" t="n"/>
-      <c r="L2" s="40" t="n"/>
-      <c r="M2" s="40" t="n"/>
-      <c r="N2" s="40" t="n"/>
-      <c r="O2" s="40" t="n"/>
+      <c r="K2" s="58" t="n"/>
+      <c r="L2" s="59" t="n"/>
+      <c r="M2" s="59" t="n"/>
+      <c r="N2" s="59" t="n"/>
+      <c r="O2" s="59" t="n"/>
+      <c r="P2" s="56" t="n"/>
+      <c r="Q2" s="56" t="n"/>
+      <c r="R2" s="56" t="n"/>
+      <c r="S2" s="56" t="n"/>
     </row>
     <row r="3" ht="16" customHeight="1">
-      <c r="A3" s="41" t="inlineStr">
+      <c r="A3" s="60" t="inlineStr">
         <is>
           <t>Модель изделия: XXX</t>
         </is>
       </c>
-      <c r="B3" s="35" t="n"/>
-      <c r="C3" s="35" t="n"/>
-      <c r="D3" s="42" t="inlineStr">
+      <c r="B3" s="61" t="n"/>
+      <c r="C3" s="61" t="n"/>
+      <c r="D3" s="61" t="inlineStr">
         <is>
           <t>Версия:</t>
         </is>
       </c>
-      <c r="E3" s="35" t="n"/>
-      <c r="F3" s="35" t="n"/>
-      <c r="G3" s="35" t="n"/>
-      <c r="H3" s="35" t="n"/>
-      <c r="I3" s="39" t="inlineStr">
+      <c r="E3" s="61" t="n"/>
+      <c r="F3" s="61" t="n"/>
+      <c r="G3" s="61" t="n"/>
+      <c r="H3" s="61" t="n"/>
+      <c r="I3" s="58" t="inlineStr">
         <is>
           <t>Проверил:</t>
         </is>
       </c>
-      <c r="J3" s="39" t="inlineStr">
+      <c r="J3" s="58" t="inlineStr">
         <is>
           <t>Дата:</t>
         </is>
       </c>
-      <c r="K3" s="34" t="n"/>
-      <c r="L3" s="40" t="n"/>
-      <c r="M3" s="40" t="n"/>
-      <c r="N3" s="40" t="n"/>
-      <c r="O3" s="40" t="n"/>
+      <c r="K3" s="58" t="n"/>
+      <c r="L3" s="59" t="n"/>
+      <c r="M3" s="59" t="n"/>
+      <c r="N3" s="59" t="n"/>
+      <c r="O3" s="59" t="n"/>
+      <c r="P3" s="56" t="n"/>
+      <c r="Q3" s="56" t="n"/>
+      <c r="R3" s="56" t="n"/>
+      <c r="S3" s="56" t="n"/>
     </row>
     <row r="4" ht="16" customHeight="1">
-      <c r="A4" s="40" t="n"/>
-      <c r="B4" s="40" t="n"/>
-      <c r="C4" s="40" t="n"/>
-      <c r="D4" s="40" t="n"/>
-      <c r="E4" s="40" t="n"/>
-      <c r="F4" s="40" t="n"/>
-      <c r="G4" s="40" t="n"/>
-      <c r="H4" s="40" t="n"/>
-      <c r="I4" s="39" t="inlineStr">
+      <c r="A4" s="59" t="n"/>
+      <c r="B4" s="59" t="n"/>
+      <c r="C4" s="59" t="n"/>
+      <c r="D4" s="59" t="n"/>
+      <c r="E4" s="59" t="n"/>
+      <c r="F4" s="59" t="n"/>
+      <c r="G4" s="59" t="n"/>
+      <c r="H4" s="59" t="n"/>
+      <c r="I4" s="58" t="inlineStr">
         <is>
           <t>Утвердил:</t>
         </is>
       </c>
-      <c r="J4" s="39" t="inlineStr">
+      <c r="J4" s="58" t="inlineStr">
         <is>
           <t>Дата:</t>
         </is>
       </c>
-      <c r="K4" s="34" t="n"/>
-      <c r="L4" s="40" t="n"/>
-      <c r="M4" s="40" t="n"/>
-      <c r="N4" s="40" t="n"/>
-      <c r="O4" s="40" t="n"/>
+      <c r="K4" s="58" t="n"/>
+      <c r="L4" s="59" t="n"/>
+      <c r="M4" s="59" t="n"/>
+      <c r="N4" s="59" t="n"/>
+      <c r="O4" s="59" t="n"/>
+      <c r="P4" s="56" t="n"/>
+      <c r="Q4" s="56" t="n"/>
+      <c r="R4" s="56" t="n"/>
+      <c r="S4" s="56" t="n"/>
     </row>
     <row r="5" ht="16" customHeight="1">
-      <c r="A5" s="39" t="n"/>
-      <c r="B5" s="39" t="n"/>
-      <c r="C5" s="39" t="n"/>
-      <c r="D5" s="39" t="n"/>
-      <c r="E5" s="39" t="n"/>
-      <c r="F5" s="39" t="n"/>
-      <c r="G5" s="39" t="n"/>
-      <c r="H5" s="39" t="n"/>
-      <c r="I5" s="39" t="inlineStr">
+      <c r="A5" s="58" t="n"/>
+      <c r="B5" s="58" t="n"/>
+      <c r="C5" s="58" t="n"/>
+      <c r="D5" s="58" t="n"/>
+      <c r="E5" s="58" t="n"/>
+      <c r="F5" s="58" t="n"/>
+      <c r="G5" s="58" t="n"/>
+      <c r="H5" s="58" t="n"/>
+      <c r="I5" s="58" t="inlineStr">
         <is>
           <t>Номер таблицы:</t>
         </is>
       </c>
-      <c r="J5" s="34" t="n"/>
-      <c r="K5" s="34" t="n"/>
-      <c r="L5" s="40" t="n"/>
-      <c r="M5" s="40" t="n"/>
-      <c r="N5" s="40" t="n"/>
-      <c r="O5" s="40" t="n"/>
+      <c r="J5" s="58" t="n"/>
+      <c r="K5" s="58" t="n"/>
+      <c r="L5" s="59" t="n"/>
+      <c r="M5" s="59" t="n"/>
+      <c r="N5" s="59" t="n"/>
+      <c r="O5" s="59" t="n"/>
+      <c r="P5" s="56" t="n"/>
+      <c r="Q5" s="56" t="n"/>
+      <c r="R5" s="56" t="n"/>
+      <c r="S5" s="56" t="n"/>
     </row>
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="43" t="inlineStr">
@@ -1374,6 +1436,10 @@
           <t>Путь</t>
         </is>
       </c>
+      <c r="P6" s="56" t="n"/>
+      <c r="Q6" s="56" t="n"/>
+      <c r="R6" s="56" t="n"/>
+      <c r="S6" s="56" t="n"/>
     </row>
     <row r="7" ht="20" customFormat="1" customHeight="1" s="15">
       <c r="A7" s="44" t="n"/>
@@ -1390,7 +1456,11 @@
       <c r="L7" s="45" t="n"/>
       <c r="M7" s="45" t="n"/>
       <c r="N7" s="45" t="n"/>
-      <c r="O7" s="46" t="n"/>
+      <c r="O7" s="62" t="n"/>
+      <c r="P7" s="56" t="n"/>
+      <c r="Q7" s="56" t="n"/>
+      <c r="R7" s="56" t="n"/>
+      <c r="S7" s="56" t="n"/>
     </row>
     <row r="8" ht="20" customFormat="1" customHeight="1" s="15">
       <c r="A8" s="44" t="n"/>
@@ -1407,7 +1477,11 @@
       <c r="L8" s="45" t="n"/>
       <c r="M8" s="45" t="n"/>
       <c r="N8" s="45" t="n"/>
-      <c r="O8" s="46" t="n"/>
+      <c r="O8" s="62" t="n"/>
+      <c r="P8" s="56" t="n"/>
+      <c r="Q8" s="56" t="n"/>
+      <c r="R8" s="56" t="n"/>
+      <c r="S8" s="56" t="n"/>
     </row>
     <row r="9" ht="20" customFormat="1" customHeight="1" s="15">
       <c r="A9" s="44" t="n"/>
@@ -1424,7 +1498,11 @@
       <c r="L9" s="45" t="n"/>
       <c r="M9" s="45" t="n"/>
       <c r="N9" s="45" t="n"/>
-      <c r="O9" s="46" t="n"/>
+      <c r="O9" s="62" t="n"/>
+      <c r="P9" s="56" t="n"/>
+      <c r="Q9" s="56" t="n"/>
+      <c r="R9" s="56" t="n"/>
+      <c r="S9" s="56" t="n"/>
     </row>
     <row r="10" ht="20" customFormat="1" customHeight="1" s="15">
       <c r="A10" s="44" t="n"/>
@@ -1441,7 +1519,11 @@
       <c r="L10" s="45" t="n"/>
       <c r="M10" s="45" t="n"/>
       <c r="N10" s="45" t="n"/>
-      <c r="O10" s="46" t="n"/>
+      <c r="O10" s="62" t="n"/>
+      <c r="P10" s="56" t="n"/>
+      <c r="Q10" s="56" t="n"/>
+      <c r="R10" s="56" t="n"/>
+      <c r="S10" s="56" t="n"/>
     </row>
     <row r="11" ht="20" customFormat="1" customHeight="1" s="15">
       <c r="A11" s="44" t="n"/>
@@ -1458,7 +1540,11 @@
       <c r="L11" s="45" t="n"/>
       <c r="M11" s="45" t="n"/>
       <c r="N11" s="45" t="n"/>
-      <c r="O11" s="46" t="n"/>
+      <c r="O11" s="62" t="n"/>
+      <c r="P11" s="56" t="n"/>
+      <c r="Q11" s="56" t="n"/>
+      <c r="R11" s="56" t="n"/>
+      <c r="S11" s="56" t="n"/>
     </row>
     <row r="12" ht="20" customFormat="1" customHeight="1" s="15">
       <c r="A12" s="44" t="n"/>
@@ -1475,7 +1561,11 @@
       <c r="L12" s="45" t="n"/>
       <c r="M12" s="45" t="n"/>
       <c r="N12" s="45" t="n"/>
-      <c r="O12" s="46" t="n"/>
+      <c r="O12" s="62" t="n"/>
+      <c r="P12" s="56" t="n"/>
+      <c r="Q12" s="56" t="n"/>
+      <c r="R12" s="56" t="n"/>
+      <c r="S12" s="56" t="n"/>
     </row>
     <row r="13" ht="20" customFormat="1" customHeight="1" s="15">
       <c r="A13" s="44" t="n"/>
@@ -1492,7 +1582,11 @@
       <c r="L13" s="45" t="n"/>
       <c r="M13" s="45" t="n"/>
       <c r="N13" s="45" t="n"/>
-      <c r="O13" s="46" t="n"/>
+      <c r="O13" s="62" t="n"/>
+      <c r="P13" s="56" t="n"/>
+      <c r="Q13" s="56" t="n"/>
+      <c r="R13" s="56" t="n"/>
+      <c r="S13" s="56" t="n"/>
     </row>
     <row r="14" ht="20" customFormat="1" customHeight="1" s="15">
       <c r="A14" s="44" t="n"/>
@@ -1509,7 +1603,11 @@
       <c r="L14" s="45" t="n"/>
       <c r="M14" s="45" t="n"/>
       <c r="N14" s="45" t="n"/>
-      <c r="O14" s="46" t="n"/>
+      <c r="O14" s="62" t="n"/>
+      <c r="P14" s="56" t="n"/>
+      <c r="Q14" s="56" t="n"/>
+      <c r="R14" s="56" t="n"/>
+      <c r="S14" s="56" t="n"/>
     </row>
     <row r="15" ht="20" customFormat="1" customHeight="1" s="15">
       <c r="A15" s="44" t="n"/>
@@ -1526,7 +1624,11 @@
       <c r="L15" s="45" t="n"/>
       <c r="M15" s="45" t="n"/>
       <c r="N15" s="45" t="n"/>
-      <c r="O15" s="46" t="n"/>
+      <c r="O15" s="62" t="n"/>
+      <c r="P15" s="56" t="n"/>
+      <c r="Q15" s="56" t="n"/>
+      <c r="R15" s="56" t="n"/>
+      <c r="S15" s="56" t="n"/>
     </row>
     <row r="16" ht="20" customFormat="1" customHeight="1" s="15">
       <c r="A16" s="44" t="n"/>
@@ -1543,7 +1645,11 @@
       <c r="L16" s="45" t="n"/>
       <c r="M16" s="45" t="n"/>
       <c r="N16" s="45" t="n"/>
-      <c r="O16" s="46" t="n"/>
+      <c r="O16" s="62" t="n"/>
+      <c r="P16" s="56" t="n"/>
+      <c r="Q16" s="56" t="n"/>
+      <c r="R16" s="56" t="n"/>
+      <c r="S16" s="56" t="n"/>
     </row>
     <row r="17" ht="20" customFormat="1" customHeight="1" s="15">
       <c r="A17" s="44" t="n"/>
@@ -1560,7 +1666,11 @@
       <c r="L17" s="45" t="n"/>
       <c r="M17" s="45" t="n"/>
       <c r="N17" s="45" t="n"/>
-      <c r="O17" s="46" t="n"/>
+      <c r="O17" s="62" t="n"/>
+      <c r="P17" s="56" t="n"/>
+      <c r="Q17" s="56" t="n"/>
+      <c r="R17" s="56" t="n"/>
+      <c r="S17" s="56" t="n"/>
     </row>
     <row r="18" ht="20" customFormat="1" customHeight="1" s="15">
       <c r="A18" s="44" t="n"/>
@@ -1577,7 +1687,11 @@
       <c r="L18" s="45" t="n"/>
       <c r="M18" s="45" t="n"/>
       <c r="N18" s="45" t="n"/>
-      <c r="O18" s="46" t="n"/>
+      <c r="O18" s="62" t="n"/>
+      <c r="P18" s="56" t="n"/>
+      <c r="Q18" s="56" t="n"/>
+      <c r="R18" s="56" t="n"/>
+      <c r="S18" s="56" t="n"/>
     </row>
     <row r="19" ht="20" customFormat="1" customHeight="1" s="15">
       <c r="A19" s="44" t="n"/>
@@ -1594,7 +1708,11 @@
       <c r="L19" s="45" t="n"/>
       <c r="M19" s="45" t="n"/>
       <c r="N19" s="45" t="n"/>
-      <c r="O19" s="46" t="n"/>
+      <c r="O19" s="62" t="n"/>
+      <c r="P19" s="56" t="n"/>
+      <c r="Q19" s="56" t="n"/>
+      <c r="R19" s="56" t="n"/>
+      <c r="S19" s="56" t="n"/>
     </row>
     <row r="20" ht="20" customFormat="1" customHeight="1" s="15">
       <c r="A20" s="44" t="n"/>
@@ -1611,7 +1729,11 @@
       <c r="L20" s="45" t="n"/>
       <c r="M20" s="45" t="n"/>
       <c r="N20" s="45" t="n"/>
-      <c r="O20" s="46" t="n"/>
+      <c r="O20" s="62" t="n"/>
+      <c r="P20" s="56" t="n"/>
+      <c r="Q20" s="56" t="n"/>
+      <c r="R20" s="56" t="n"/>
+      <c r="S20" s="56" t="n"/>
     </row>
     <row r="21" ht="20" customFormat="1" customHeight="1" s="15">
       <c r="A21" s="44" t="n"/>
@@ -1628,7 +1750,11 @@
       <c r="L21" s="45" t="n"/>
       <c r="M21" s="45" t="n"/>
       <c r="N21" s="45" t="n"/>
-      <c r="O21" s="46" t="n"/>
+      <c r="O21" s="62" t="n"/>
+      <c r="P21" s="56" t="n"/>
+      <c r="Q21" s="56" t="n"/>
+      <c r="R21" s="56" t="n"/>
+      <c r="S21" s="56" t="n"/>
     </row>
     <row r="22" ht="20" customFormat="1" customHeight="1" s="15">
       <c r="A22" s="44" t="n"/>
@@ -1645,7 +1771,11 @@
       <c r="L22" s="45" t="n"/>
       <c r="M22" s="45" t="n"/>
       <c r="N22" s="45" t="n"/>
-      <c r="O22" s="46" t="n"/>
+      <c r="O22" s="62" t="n"/>
+      <c r="P22" s="56" t="n"/>
+      <c r="Q22" s="56" t="n"/>
+      <c r="R22" s="56" t="n"/>
+      <c r="S22" s="56" t="n"/>
     </row>
     <row r="23" ht="20" customFormat="1" customHeight="1" s="15">
       <c r="A23" s="44" t="n"/>
@@ -1662,7 +1792,11 @@
       <c r="L23" s="45" t="n"/>
       <c r="M23" s="45" t="n"/>
       <c r="N23" s="45" t="n"/>
-      <c r="O23" s="46" t="n"/>
+      <c r="O23" s="62" t="n"/>
+      <c r="P23" s="56" t="n"/>
+      <c r="Q23" s="56" t="n"/>
+      <c r="R23" s="56" t="n"/>
+      <c r="S23" s="56" t="n"/>
     </row>
     <row r="24" ht="20" customFormat="1" customHeight="1" s="15">
       <c r="A24" s="44" t="n"/>
@@ -1679,7 +1813,11 @@
       <c r="L24" s="45" t="n"/>
       <c r="M24" s="45" t="n"/>
       <c r="N24" s="45" t="n"/>
-      <c r="O24" s="46" t="n"/>
+      <c r="O24" s="62" t="n"/>
+      <c r="P24" s="56" t="n"/>
+      <c r="Q24" s="56" t="n"/>
+      <c r="R24" s="56" t="n"/>
+      <c r="S24" s="56" t="n"/>
     </row>
     <row r="25" ht="20" customFormat="1" customHeight="1" s="15">
       <c r="A25" s="44" t="n"/>
@@ -1696,7 +1834,11 @@
       <c r="L25" s="45" t="n"/>
       <c r="M25" s="45" t="n"/>
       <c r="N25" s="45" t="n"/>
-      <c r="O25" s="46" t="n"/>
+      <c r="O25" s="62" t="n"/>
+      <c r="P25" s="56" t="n"/>
+      <c r="Q25" s="56" t="n"/>
+      <c r="R25" s="56" t="n"/>
+      <c r="S25" s="56" t="n"/>
     </row>
     <row r="26" ht="20" customFormat="1" customHeight="1" s="15">
       <c r="A26" s="44" t="n"/>
@@ -1713,7 +1855,11 @@
       <c r="L26" s="45" t="n"/>
       <c r="M26" s="45" t="n"/>
       <c r="N26" s="45" t="n"/>
-      <c r="O26" s="46" t="n"/>
+      <c r="O26" s="62" t="n"/>
+      <c r="P26" s="56" t="n"/>
+      <c r="Q26" s="56" t="n"/>
+      <c r="R26" s="56" t="n"/>
+      <c r="S26" s="56" t="n"/>
     </row>
     <row r="27" ht="20" customFormat="1" customHeight="1" s="15">
       <c r="A27" s="44" t="n"/>
@@ -1730,7 +1876,11 @@
       <c r="L27" s="45" t="n"/>
       <c r="M27" s="45" t="n"/>
       <c r="N27" s="45" t="n"/>
-      <c r="O27" s="46" t="n"/>
+      <c r="O27" s="62" t="n"/>
+      <c r="P27" s="56" t="n"/>
+      <c r="Q27" s="56" t="n"/>
+      <c r="R27" s="56" t="n"/>
+      <c r="S27" s="56" t="n"/>
     </row>
     <row r="28" ht="20" customFormat="1" customHeight="1" s="15">
       <c r="A28" s="44" t="n"/>
@@ -1747,7 +1897,11 @@
       <c r="L28" s="45" t="n"/>
       <c r="M28" s="45" t="n"/>
       <c r="N28" s="45" t="n"/>
-      <c r="O28" s="46" t="n"/>
+      <c r="O28" s="62" t="n"/>
+      <c r="P28" s="56" t="n"/>
+      <c r="Q28" s="56" t="n"/>
+      <c r="R28" s="56" t="n"/>
+      <c r="S28" s="56" t="n"/>
     </row>
     <row r="29" ht="20" customFormat="1" customHeight="1" s="15">
       <c r="A29" s="44" t="n"/>
@@ -1764,7 +1918,11 @@
       <c r="L29" s="45" t="n"/>
       <c r="M29" s="45" t="n"/>
       <c r="N29" s="45" t="n"/>
-      <c r="O29" s="46" t="n"/>
+      <c r="O29" s="62" t="n"/>
+      <c r="P29" s="56" t="n"/>
+      <c r="Q29" s="56" t="n"/>
+      <c r="R29" s="56" t="n"/>
+      <c r="S29" s="56" t="n"/>
     </row>
     <row r="30" ht="20" customFormat="1" customHeight="1" s="15">
       <c r="A30" s="44" t="n"/>
@@ -1781,7 +1939,11 @@
       <c r="L30" s="45" t="n"/>
       <c r="M30" s="45" t="n"/>
       <c r="N30" s="45" t="n"/>
-      <c r="O30" s="46" t="n"/>
+      <c r="O30" s="62" t="n"/>
+      <c r="P30" s="56" t="n"/>
+      <c r="Q30" s="56" t="n"/>
+      <c r="R30" s="56" t="n"/>
+      <c r="S30" s="56" t="n"/>
     </row>
     <row r="31" ht="20" customFormat="1" customHeight="1" s="15">
       <c r="A31" s="44" t="n"/>
@@ -1798,7 +1960,11 @@
       <c r="L31" s="45" t="n"/>
       <c r="M31" s="45" t="n"/>
       <c r="N31" s="45" t="n"/>
-      <c r="O31" s="46" t="n"/>
+      <c r="O31" s="62" t="n"/>
+      <c r="P31" s="56" t="n"/>
+      <c r="Q31" s="56" t="n"/>
+      <c r="R31" s="56" t="n"/>
+      <c r="S31" s="56" t="n"/>
     </row>
     <row r="32" ht="20" customFormat="1" customHeight="1" s="15">
       <c r="A32" s="44" t="n"/>
@@ -1815,7 +1981,11 @@
       <c r="L32" s="45" t="n"/>
       <c r="M32" s="45" t="n"/>
       <c r="N32" s="45" t="n"/>
-      <c r="O32" s="46" t="n"/>
+      <c r="O32" s="62" t="n"/>
+      <c r="P32" s="56" t="n"/>
+      <c r="Q32" s="56" t="n"/>
+      <c r="R32" s="56" t="n"/>
+      <c r="S32" s="56" t="n"/>
     </row>
     <row r="33" ht="20" customFormat="1" customHeight="1" s="15">
       <c r="A33" s="44" t="n"/>
@@ -1832,7 +2002,11 @@
       <c r="L33" s="45" t="n"/>
       <c r="M33" s="45" t="n"/>
       <c r="N33" s="45" t="n"/>
-      <c r="O33" s="46" t="n"/>
+      <c r="O33" s="62" t="n"/>
+      <c r="P33" s="56" t="n"/>
+      <c r="Q33" s="56" t="n"/>
+      <c r="R33" s="56" t="n"/>
+      <c r="S33" s="56" t="n"/>
     </row>
     <row r="34" ht="20" customFormat="1" customHeight="1" s="15">
       <c r="A34" s="44" t="n"/>
@@ -1849,7 +2023,11 @@
       <c r="L34" s="45" t="n"/>
       <c r="M34" s="45" t="n"/>
       <c r="N34" s="45" t="n"/>
-      <c r="O34" s="46" t="n"/>
+      <c r="O34" s="62" t="n"/>
+      <c r="P34" s="56" t="n"/>
+      <c r="Q34" s="56" t="n"/>
+      <c r="R34" s="56" t="n"/>
+      <c r="S34" s="56" t="n"/>
     </row>
     <row r="35" ht="20" customFormat="1" customHeight="1" s="15">
       <c r="A35" s="44" t="n"/>
@@ -1866,7 +2044,11 @@
       <c r="L35" s="45" t="n"/>
       <c r="M35" s="45" t="n"/>
       <c r="N35" s="45" t="n"/>
-      <c r="O35" s="46" t="n"/>
+      <c r="O35" s="62" t="n"/>
+      <c r="P35" s="56" t="n"/>
+      <c r="Q35" s="56" t="n"/>
+      <c r="R35" s="56" t="n"/>
+      <c r="S35" s="56" t="n"/>
     </row>
     <row r="36" ht="20" customFormat="1" customHeight="1" s="15">
       <c r="A36" s="44" t="n"/>
@@ -1883,7 +2065,11 @@
       <c r="L36" s="45" t="n"/>
       <c r="M36" s="45" t="n"/>
       <c r="N36" s="45" t="n"/>
-      <c r="O36" s="46" t="n"/>
+      <c r="O36" s="62" t="n"/>
+      <c r="P36" s="56" t="n"/>
+      <c r="Q36" s="56" t="n"/>
+      <c r="R36" s="56" t="n"/>
+      <c r="S36" s="56" t="n"/>
     </row>
     <row r="37" ht="20" customFormat="1" customHeight="1" s="15">
       <c r="A37" s="44" t="n"/>
@@ -1900,7 +2086,11 @@
       <c r="L37" s="45" t="n"/>
       <c r="M37" s="45" t="n"/>
       <c r="N37" s="45" t="n"/>
-      <c r="O37" s="46" t="n"/>
+      <c r="O37" s="62" t="n"/>
+      <c r="P37" s="56" t="n"/>
+      <c r="Q37" s="56" t="n"/>
+      <c r="R37" s="56" t="n"/>
+      <c r="S37" s="56" t="n"/>
     </row>
     <row r="38" ht="20" customFormat="1" customHeight="1" s="15">
       <c r="A38" s="44" t="n"/>
@@ -1917,7 +2107,11 @@
       <c r="L38" s="45" t="n"/>
       <c r="M38" s="45" t="n"/>
       <c r="N38" s="45" t="n"/>
-      <c r="O38" s="46" t="n"/>
+      <c r="O38" s="62" t="n"/>
+      <c r="P38" s="56" t="n"/>
+      <c r="Q38" s="56" t="n"/>
+      <c r="R38" s="56" t="n"/>
+      <c r="S38" s="56" t="n"/>
     </row>
     <row r="39" ht="20" customFormat="1" customHeight="1" s="15">
       <c r="A39" s="44" t="n"/>
@@ -1934,7 +2128,11 @@
       <c r="L39" s="45" t="n"/>
       <c r="M39" s="45" t="n"/>
       <c r="N39" s="45" t="n"/>
-      <c r="O39" s="46" t="n"/>
+      <c r="O39" s="62" t="n"/>
+      <c r="P39" s="56" t="n"/>
+      <c r="Q39" s="56" t="n"/>
+      <c r="R39" s="56" t="n"/>
+      <c r="S39" s="56" t="n"/>
     </row>
     <row r="40" ht="20" customFormat="1" customHeight="1" s="15">
       <c r="A40" s="44" t="n"/>
@@ -1951,7 +2149,11 @@
       <c r="L40" s="45" t="n"/>
       <c r="M40" s="45" t="n"/>
       <c r="N40" s="45" t="n"/>
-      <c r="O40" s="46" t="n"/>
+      <c r="O40" s="62" t="n"/>
+      <c r="P40" s="56" t="n"/>
+      <c r="Q40" s="56" t="n"/>
+      <c r="R40" s="56" t="n"/>
+      <c r="S40" s="56" t="n"/>
     </row>
     <row r="41" ht="20" customHeight="1">
       <c r="A41" s="44" t="n"/>
@@ -1968,7 +2170,11 @@
       <c r="L41" s="45" t="n"/>
       <c r="M41" s="45" t="n"/>
       <c r="N41" s="45" t="n"/>
-      <c r="O41" s="46" t="n"/>
+      <c r="O41" s="62" t="n"/>
+      <c r="P41" s="56" t="n"/>
+      <c r="Q41" s="56" t="n"/>
+      <c r="R41" s="56" t="n"/>
+      <c r="S41" s="56" t="n"/>
     </row>
     <row r="42" ht="20" customHeight="1">
       <c r="A42" s="44" t="n"/>
@@ -1985,7 +2191,11 @@
       <c r="L42" s="45" t="n"/>
       <c r="M42" s="45" t="n"/>
       <c r="N42" s="45" t="n"/>
-      <c r="O42" s="46" t="n"/>
+      <c r="O42" s="62" t="n"/>
+      <c r="P42" s="56" t="n"/>
+      <c r="Q42" s="56" t="n"/>
+      <c r="R42" s="56" t="n"/>
+      <c r="S42" s="56" t="n"/>
     </row>
     <row r="43" ht="20" customHeight="1">
       <c r="A43" s="44" t="n"/>
@@ -2002,7 +2212,11 @@
       <c r="L43" s="45" t="n"/>
       <c r="M43" s="45" t="n"/>
       <c r="N43" s="45" t="n"/>
-      <c r="O43" s="46" t="n"/>
+      <c r="O43" s="62" t="n"/>
+      <c r="P43" s="56" t="n"/>
+      <c r="Q43" s="56" t="n"/>
+      <c r="R43" s="56" t="n"/>
+      <c r="S43" s="56" t="n"/>
     </row>
     <row r="44" ht="20" customHeight="1">
       <c r="A44" s="44" t="n"/>
@@ -2019,7 +2233,11 @@
       <c r="L44" s="45" t="n"/>
       <c r="M44" s="45" t="n"/>
       <c r="N44" s="45" t="n"/>
-      <c r="O44" s="46" t="n"/>
+      <c r="O44" s="62" t="n"/>
+      <c r="P44" s="56" t="n"/>
+      <c r="Q44" s="56" t="n"/>
+      <c r="R44" s="56" t="n"/>
+      <c r="S44" s="56" t="n"/>
     </row>
     <row r="45" ht="20" customHeight="1">
       <c r="A45" s="44" t="n"/>
@@ -2036,7 +2254,11 @@
       <c r="L45" s="45" t="n"/>
       <c r="M45" s="45" t="n"/>
       <c r="N45" s="45" t="n"/>
-      <c r="O45" s="46" t="n"/>
+      <c r="O45" s="62" t="n"/>
+      <c r="P45" s="56" t="n"/>
+      <c r="Q45" s="56" t="n"/>
+      <c r="R45" s="56" t="n"/>
+      <c r="S45" s="56" t="n"/>
     </row>
     <row r="46" ht="20" customHeight="1">
       <c r="A46" s="44" t="n"/>
@@ -2053,11 +2275,11 @@
       <c r="L46" s="45" t="n"/>
       <c r="M46" s="45" t="n"/>
       <c r="N46" s="45" t="n"/>
-      <c r="O46" s="46" t="n"/>
-      <c r="P46" s="9" t="n"/>
-      <c r="Q46" s="9" t="n"/>
-      <c r="R46" s="3" t="n"/>
-      <c r="S46" s="36" t="n"/>
+      <c r="O46" s="62" t="n"/>
+      <c r="P46" s="63" t="n"/>
+      <c r="Q46" s="63" t="n"/>
+      <c r="R46" s="64" t="n"/>
+      <c r="S46" s="65" t="n"/>
     </row>
     <row r="47" ht="20" customHeight="1">
       <c r="A47" s="44" t="n"/>
@@ -2074,7 +2296,11 @@
       <c r="L47" s="45" t="n"/>
       <c r="M47" s="45" t="n"/>
       <c r="N47" s="45" t="n"/>
-      <c r="O47" s="46" t="n"/>
+      <c r="O47" s="62" t="n"/>
+      <c r="P47" s="56" t="n"/>
+      <c r="Q47" s="56" t="n"/>
+      <c r="R47" s="56" t="n"/>
+      <c r="S47" s="56" t="n"/>
     </row>
     <row r="48" ht="20" customHeight="1">
       <c r="A48" s="44" t="n"/>
@@ -2091,7 +2317,11 @@
       <c r="L48" s="45" t="n"/>
       <c r="M48" s="45" t="n"/>
       <c r="N48" s="45" t="n"/>
-      <c r="O48" s="46" t="n"/>
+      <c r="O48" s="62" t="n"/>
+      <c r="P48" s="56" t="n"/>
+      <c r="Q48" s="56" t="n"/>
+      <c r="R48" s="56" t="n"/>
+      <c r="S48" s="56" t="n"/>
     </row>
     <row r="49" ht="20" customHeight="1">
       <c r="A49" s="44" t="n"/>
@@ -2108,7 +2338,11 @@
       <c r="L49" s="45" t="n"/>
       <c r="M49" s="45" t="n"/>
       <c r="N49" s="45" t="n"/>
-      <c r="O49" s="46" t="n"/>
+      <c r="O49" s="62" t="n"/>
+      <c r="P49" s="56" t="n"/>
+      <c r="Q49" s="56" t="n"/>
+      <c r="R49" s="56" t="n"/>
+      <c r="S49" s="56" t="n"/>
     </row>
     <row r="50" ht="20" customHeight="1">
       <c r="A50" s="44" t="n"/>
@@ -2125,7 +2359,11 @@
       <c r="L50" s="45" t="n"/>
       <c r="M50" s="45" t="n"/>
       <c r="N50" s="45" t="n"/>
-      <c r="O50" s="46" t="n"/>
+      <c r="O50" s="62" t="n"/>
+      <c r="P50" s="56" t="n"/>
+      <c r="Q50" s="56" t="n"/>
+      <c r="R50" s="56" t="n"/>
+      <c r="S50" s="56" t="n"/>
     </row>
     <row r="51" ht="20" customHeight="1">
       <c r="A51" s="44" t="n"/>
@@ -2142,7 +2380,11 @@
       <c r="L51" s="45" t="n"/>
       <c r="M51" s="45" t="n"/>
       <c r="N51" s="45" t="n"/>
-      <c r="O51" s="46" t="n"/>
+      <c r="O51" s="62" t="n"/>
+      <c r="P51" s="56" t="n"/>
+      <c r="Q51" s="56" t="n"/>
+      <c r="R51" s="56" t="n"/>
+      <c r="S51" s="56" t="n"/>
     </row>
     <row r="52" ht="20" customHeight="1">
       <c r="A52" s="44" t="n"/>
@@ -2159,7 +2401,11 @@
       <c r="L52" s="45" t="n"/>
       <c r="M52" s="45" t="n"/>
       <c r="N52" s="45" t="n"/>
-      <c r="O52" s="46" t="n"/>
+      <c r="O52" s="62" t="n"/>
+      <c r="P52" s="56" t="n"/>
+      <c r="Q52" s="56" t="n"/>
+      <c r="R52" s="56" t="n"/>
+      <c r="S52" s="56" t="n"/>
     </row>
     <row r="53" ht="20" customHeight="1">
       <c r="A53" s="44" t="n"/>
@@ -2176,7 +2422,11 @@
       <c r="L53" s="45" t="n"/>
       <c r="M53" s="45" t="n"/>
       <c r="N53" s="45" t="n"/>
-      <c r="O53" s="46" t="n"/>
+      <c r="O53" s="62" t="n"/>
+      <c r="P53" s="56" t="n"/>
+      <c r="Q53" s="56" t="n"/>
+      <c r="R53" s="56" t="n"/>
+      <c r="S53" s="56" t="n"/>
     </row>
     <row r="54" ht="20" customHeight="1">
       <c r="A54" s="44" t="n"/>
@@ -2193,11 +2443,11 @@
       <c r="L54" s="45" t="n"/>
       <c r="M54" s="45" t="n"/>
       <c r="N54" s="45" t="n"/>
-      <c r="O54" s="46" t="n"/>
-      <c r="P54" s="9" t="n"/>
-      <c r="Q54" s="9" t="n"/>
-      <c r="R54" s="3" t="n"/>
-      <c r="S54" s="36" t="n"/>
+      <c r="O54" s="62" t="n"/>
+      <c r="P54" s="63" t="n"/>
+      <c r="Q54" s="63" t="n"/>
+      <c r="R54" s="64" t="n"/>
+      <c r="S54" s="65" t="n"/>
     </row>
     <row r="55" ht="20" customHeight="1">
       <c r="A55" s="44" t="n"/>
@@ -2214,7 +2464,11 @@
       <c r="L55" s="45" t="n"/>
       <c r="M55" s="45" t="n"/>
       <c r="N55" s="45" t="n"/>
-      <c r="O55" s="46" t="n"/>
+      <c r="O55" s="62" t="n"/>
+      <c r="P55" s="56" t="n"/>
+      <c r="Q55" s="56" t="n"/>
+      <c r="R55" s="56" t="n"/>
+      <c r="S55" s="56" t="n"/>
     </row>
     <row r="56" ht="20" customHeight="1">
       <c r="A56" s="44" t="n"/>
@@ -2231,7 +2485,11 @@
       <c r="L56" s="45" t="n"/>
       <c r="M56" s="45" t="n"/>
       <c r="N56" s="45" t="n"/>
-      <c r="O56" s="46" t="n"/>
+      <c r="O56" s="62" t="n"/>
+      <c r="P56" s="56" t="n"/>
+      <c r="Q56" s="56" t="n"/>
+      <c r="R56" s="56" t="n"/>
+      <c r="S56" s="56" t="n"/>
     </row>
     <row r="57" ht="20" customHeight="1">
       <c r="A57" s="44" t="n"/>
@@ -2248,7 +2506,11 @@
       <c r="L57" s="45" t="n"/>
       <c r="M57" s="45" t="n"/>
       <c r="N57" s="45" t="n"/>
-      <c r="O57" s="46" t="n"/>
+      <c r="O57" s="62" t="n"/>
+      <c r="P57" s="56" t="n"/>
+      <c r="Q57" s="56" t="n"/>
+      <c r="R57" s="56" t="n"/>
+      <c r="S57" s="56" t="n"/>
     </row>
     <row r="58" ht="20" customHeight="1">
       <c r="A58" s="44" t="n"/>
@@ -2265,11 +2527,11 @@
       <c r="L58" s="45" t="n"/>
       <c r="M58" s="45" t="n"/>
       <c r="N58" s="45" t="n"/>
-      <c r="O58" s="46" t="n"/>
-      <c r="P58" s="9" t="n"/>
-      <c r="Q58" s="9" t="n"/>
-      <c r="R58" s="3" t="n"/>
-      <c r="S58" s="36" t="n"/>
+      <c r="O58" s="62" t="n"/>
+      <c r="P58" s="63" t="n"/>
+      <c r="Q58" s="63" t="n"/>
+      <c r="R58" s="64" t="n"/>
+      <c r="S58" s="65" t="n"/>
     </row>
     <row r="59" ht="20" customHeight="1">
       <c r="A59" s="44" t="n"/>
@@ -2286,7 +2548,11 @@
       <c r="L59" s="45" t="n"/>
       <c r="M59" s="45" t="n"/>
       <c r="N59" s="45" t="n"/>
-      <c r="O59" s="46" t="n"/>
+      <c r="O59" s="62" t="n"/>
+      <c r="P59" s="56" t="n"/>
+      <c r="Q59" s="56" t="n"/>
+      <c r="R59" s="56" t="n"/>
+      <c r="S59" s="56" t="n"/>
     </row>
     <row r="60" ht="20" customHeight="1">
       <c r="A60" s="44" t="n"/>
@@ -2303,7 +2569,11 @@
       <c r="L60" s="45" t="n"/>
       <c r="M60" s="45" t="n"/>
       <c r="N60" s="45" t="n"/>
-      <c r="O60" s="46" t="n"/>
+      <c r="O60" s="62" t="n"/>
+      <c r="P60" s="56" t="n"/>
+      <c r="Q60" s="56" t="n"/>
+      <c r="R60" s="56" t="n"/>
+      <c r="S60" s="56" t="n"/>
     </row>
     <row r="61" ht="20" customHeight="1">
       <c r="A61" s="44" t="n"/>
@@ -2320,7 +2590,11 @@
       <c r="L61" s="45" t="n"/>
       <c r="M61" s="45" t="n"/>
       <c r="N61" s="45" t="n"/>
-      <c r="O61" s="46" t="n"/>
+      <c r="O61" s="62" t="n"/>
+      <c r="P61" s="56" t="n"/>
+      <c r="Q61" s="56" t="n"/>
+      <c r="R61" s="56" t="n"/>
+      <c r="S61" s="56" t="n"/>
     </row>
     <row r="62" ht="20" customHeight="1">
       <c r="A62" s="44" t="n"/>
@@ -2337,7 +2611,11 @@
       <c r="L62" s="45" t="n"/>
       <c r="M62" s="45" t="n"/>
       <c r="N62" s="45" t="n"/>
-      <c r="O62" s="46" t="n"/>
+      <c r="O62" s="62" t="n"/>
+      <c r="P62" s="56" t="n"/>
+      <c r="Q62" s="56" t="n"/>
+      <c r="R62" s="56" t="n"/>
+      <c r="S62" s="56" t="n"/>
     </row>
     <row r="63" ht="20" customHeight="1">
       <c r="A63" s="44" t="n"/>
@@ -2354,7 +2632,11 @@
       <c r="L63" s="45" t="n"/>
       <c r="M63" s="45" t="n"/>
       <c r="N63" s="45" t="n"/>
-      <c r="O63" s="46" t="n"/>
+      <c r="O63" s="62" t="n"/>
+      <c r="P63" s="56" t="n"/>
+      <c r="Q63" s="56" t="n"/>
+      <c r="R63" s="56" t="n"/>
+      <c r="S63" s="56" t="n"/>
     </row>
     <row r="64" ht="20" customHeight="1">
       <c r="A64" s="44" t="n"/>
@@ -2371,7 +2653,11 @@
       <c r="L64" s="45" t="n"/>
       <c r="M64" s="45" t="n"/>
       <c r="N64" s="45" t="n"/>
-      <c r="O64" s="46" t="n"/>
+      <c r="O64" s="62" t="n"/>
+      <c r="P64" s="56" t="n"/>
+      <c r="Q64" s="56" t="n"/>
+      <c r="R64" s="56" t="n"/>
+      <c r="S64" s="56" t="n"/>
     </row>
     <row r="65" ht="20" customHeight="1">
       <c r="A65" s="44" t="n"/>
@@ -2388,7 +2674,11 @@
       <c r="L65" s="45" t="n"/>
       <c r="M65" s="45" t="n"/>
       <c r="N65" s="45" t="n"/>
-      <c r="O65" s="46" t="n"/>
+      <c r="O65" s="62" t="n"/>
+      <c r="P65" s="56" t="n"/>
+      <c r="Q65" s="56" t="n"/>
+      <c r="R65" s="56" t="n"/>
+      <c r="S65" s="56" t="n"/>
     </row>
     <row r="66" ht="20" customHeight="1">
       <c r="A66" s="44" t="n"/>
@@ -2405,7 +2695,11 @@
       <c r="L66" s="45" t="n"/>
       <c r="M66" s="45" t="n"/>
       <c r="N66" s="45" t="n"/>
-      <c r="O66" s="46" t="n"/>
+      <c r="O66" s="62" t="n"/>
+      <c r="P66" s="56" t="n"/>
+      <c r="Q66" s="56" t="n"/>
+      <c r="R66" s="56" t="n"/>
+      <c r="S66" s="56" t="n"/>
     </row>
     <row r="67" ht="20" customHeight="1">
       <c r="A67" s="44" t="n"/>
@@ -2422,7 +2716,11 @@
       <c r="L67" s="45" t="n"/>
       <c r="M67" s="45" t="n"/>
       <c r="N67" s="45" t="n"/>
-      <c r="O67" s="46" t="n"/>
+      <c r="O67" s="62" t="n"/>
+      <c r="P67" s="56" t="n"/>
+      <c r="Q67" s="56" t="n"/>
+      <c r="R67" s="56" t="n"/>
+      <c r="S67" s="56" t="n"/>
     </row>
     <row r="68" ht="20" customHeight="1">
       <c r="A68" s="44" t="n"/>
@@ -2439,7 +2737,11 @@
       <c r="L68" s="45" t="n"/>
       <c r="M68" s="45" t="n"/>
       <c r="N68" s="45" t="n"/>
-      <c r="O68" s="46" t="n"/>
+      <c r="O68" s="62" t="n"/>
+      <c r="P68" s="56" t="n"/>
+      <c r="Q68" s="56" t="n"/>
+      <c r="R68" s="56" t="n"/>
+      <c r="S68" s="56" t="n"/>
     </row>
     <row r="69" ht="20" customHeight="1">
       <c r="A69" s="44" t="n"/>
@@ -2456,7 +2758,11 @@
       <c r="L69" s="45" t="n"/>
       <c r="M69" s="45" t="n"/>
       <c r="N69" s="45" t="n"/>
-      <c r="O69" s="46" t="n"/>
+      <c r="O69" s="62" t="n"/>
+      <c r="P69" s="56" t="n"/>
+      <c r="Q69" s="56" t="n"/>
+      <c r="R69" s="56" t="n"/>
+      <c r="S69" s="56" t="n"/>
     </row>
     <row r="70" ht="20" customHeight="1">
       <c r="A70" s="44" t="n"/>
@@ -2473,7 +2779,11 @@
       <c r="L70" s="45" t="n"/>
       <c r="M70" s="45" t="n"/>
       <c r="N70" s="45" t="n"/>
-      <c r="O70" s="46" t="n"/>
+      <c r="O70" s="62" t="n"/>
+      <c r="P70" s="56" t="n"/>
+      <c r="Q70" s="56" t="n"/>
+      <c r="R70" s="56" t="n"/>
+      <c r="S70" s="56" t="n"/>
     </row>
     <row r="71" ht="20" customHeight="1">
       <c r="A71" s="44" t="n"/>
@@ -2490,73 +2800,95 @@
       <c r="L71" s="45" t="n"/>
       <c r="M71" s="45" t="n"/>
       <c r="N71" s="45" t="n"/>
-      <c r="O71" s="46" t="n"/>
+      <c r="O71" s="62" t="n"/>
+      <c r="P71" s="56" t="n"/>
+      <c r="Q71" s="56" t="n"/>
+      <c r="R71" s="56" t="n"/>
+      <c r="S71" s="56" t="n"/>
     </row>
     <row r="72" ht="20" customHeight="1">
       <c r="A72" s="44" t="n"/>
       <c r="B72" s="45" t="n"/>
       <c r="C72" s="45" t="n"/>
-      <c r="D72" s="49" t="n"/>
-      <c r="E72" s="50" t="n"/>
+      <c r="D72" s="45" t="n"/>
+      <c r="E72" s="45" t="n"/>
       <c r="F72" s="45" t="n"/>
-      <c r="G72" s="50" t="n"/>
+      <c r="G72" s="44" t="n"/>
       <c r="H72" s="45" t="n"/>
-      <c r="I72" s="49" t="n"/>
-      <c r="J72" s="49" t="n"/>
-      <c r="K72" s="50" t="n"/>
+      <c r="I72" s="45" t="n"/>
+      <c r="J72" s="44" t="n"/>
+      <c r="K72" s="45" t="n"/>
       <c r="L72" s="45" t="n"/>
       <c r="M72" s="45" t="n"/>
       <c r="N72" s="45" t="n"/>
-      <c r="O72" s="46" t="n"/>
+      <c r="O72" s="62" t="n"/>
+      <c r="P72" s="56" t="n"/>
+      <c r="Q72" s="56" t="n"/>
+      <c r="R72" s="56" t="n"/>
+      <c r="S72" s="56" t="n"/>
     </row>
     <row r="73" ht="20" customHeight="1">
       <c r="A73" s="44" t="n"/>
       <c r="B73" s="48" t="n"/>
-      <c r="C73" s="51" t="n"/>
-      <c r="E73" s="52" t="n"/>
-      <c r="F73" s="53" t="n"/>
-      <c r="G73" s="54" t="n"/>
-      <c r="H73" s="53" t="n"/>
-      <c r="I73" s="55" t="n"/>
-      <c r="J73" s="55" t="n"/>
-      <c r="K73" s="54" t="n"/>
+      <c r="C73" s="45" t="n"/>
+      <c r="D73" s="45" t="n"/>
+      <c r="E73" s="45" t="n"/>
+      <c r="F73" s="45" t="n"/>
+      <c r="G73" s="44" t="n"/>
+      <c r="H73" s="45" t="n"/>
+      <c r="I73" s="45" t="n"/>
+      <c r="J73" s="44" t="n"/>
+      <c r="K73" s="45" t="n"/>
       <c r="L73" s="45" t="n"/>
       <c r="M73" s="45" t="n"/>
       <c r="N73" s="45" t="n"/>
-      <c r="O73" s="46" t="n"/>
+      <c r="O73" s="62" t="n"/>
+      <c r="P73" s="56" t="n"/>
+      <c r="Q73" s="56" t="n"/>
+      <c r="R73" s="56" t="n"/>
+      <c r="S73" s="56" t="n"/>
     </row>
     <row r="74" ht="20" customHeight="1">
       <c r="A74" s="44" t="n"/>
       <c r="B74" s="45" t="n"/>
-      <c r="C74" s="51" t="n"/>
-      <c r="E74" s="52" t="n"/>
+      <c r="C74" s="45" t="n"/>
+      <c r="D74" s="45" t="n"/>
+      <c r="E74" s="45" t="n"/>
       <c r="F74" s="45" t="n"/>
-      <c r="G74" s="50" t="n"/>
+      <c r="G74" s="44" t="n"/>
       <c r="H74" s="45" t="n"/>
-      <c r="I74" s="49" t="n"/>
-      <c r="J74" s="49" t="n"/>
-      <c r="K74" s="50" t="n"/>
+      <c r="I74" s="45" t="n"/>
+      <c r="J74" s="44" t="n"/>
+      <c r="K74" s="45" t="n"/>
       <c r="L74" s="45" t="n"/>
       <c r="M74" s="45" t="n"/>
       <c r="N74" s="45" t="n"/>
-      <c r="O74" s="46" t="n"/>
+      <c r="O74" s="62" t="n"/>
+      <c r="P74" s="56" t="n"/>
+      <c r="Q74" s="56" t="n"/>
+      <c r="R74" s="56" t="n"/>
+      <c r="S74" s="56" t="n"/>
     </row>
     <row r="75" ht="20" customHeight="1">
       <c r="A75" s="44" t="n"/>
       <c r="B75" s="45" t="n"/>
-      <c r="C75" s="53" t="n"/>
-      <c r="D75" s="55" t="n"/>
-      <c r="E75" s="54" t="n"/>
-      <c r="F75" s="53" t="n"/>
-      <c r="G75" s="54" t="n"/>
-      <c r="H75" s="53" t="n"/>
-      <c r="I75" s="55" t="n"/>
-      <c r="J75" s="55" t="n"/>
-      <c r="K75" s="54" t="n"/>
+      <c r="C75" s="45" t="n"/>
+      <c r="D75" s="45" t="n"/>
+      <c r="E75" s="45" t="n"/>
+      <c r="F75" s="45" t="n"/>
+      <c r="G75" s="44" t="n"/>
+      <c r="H75" s="45" t="n"/>
+      <c r="I75" s="45" t="n"/>
+      <c r="J75" s="44" t="n"/>
+      <c r="K75" s="45" t="n"/>
       <c r="L75" s="45" t="n"/>
       <c r="M75" s="45" t="n"/>
       <c r="N75" s="45" t="n"/>
-      <c r="O75" s="46" t="n"/>
+      <c r="O75" s="62" t="n"/>
+      <c r="P75" s="56" t="n"/>
+      <c r="Q75" s="56" t="n"/>
+      <c r="R75" s="56" t="n"/>
+      <c r="S75" s="56" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="14">
@@ -2577,6 +2909,6 @@
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.1968503937007874" right="0.1968503937007874" top="0.1968503937007874" bottom="0.1968503937007874" header="0.1968503937007874" footer="0.3149606299212598"/>
-  <pageSetup orientation="portrait" paperSize="9"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix(bom-template): purge CJK fonts at the styles.xml level (absolute, incl. merged shadow cells)
The per-cell openpyxl pass could not reach merged-range shadow cells (MergedCell
font assignment is silently ignored) nor stale entries in the workbook font
table, so 58 cells (B1:K3, footer 72:75) kept the 宋/SimSun font even though
they never render. Re-merging in openpyxl re-introduces those shadows from the
old style, so unmerge/re-merge does not help.

Fix at the source: after save(), rewrite xl/styles.xml so every <font> whose
name contains a CJK codepoint becomes Arial, and drop charset="134" (GB2312)
hints that make Excel substitute a CJK fallback. Result: 0 CJK font names in the
file (verified in raw styles.xml), 14 merges + 16 anchors + landscape/print-area
all preserved.
</commit_message>
<xml_diff>
--- a/Шаблоны спецификации/bom_шаблон.xlsx
+++ b/Шаблоны спецификации/bom_шаблон.xlsx
@@ -39,133 +39,115 @@
   </numFmts>
   <fonts count="31">
     <font>
-      <name val="宋体"/>
-      <charset val="134"/>
+      <name val="Arial"/>
       <sz val="12"/>
     </font>
     <font>
-      <name val="宋体"/>
-      <charset val="134"/>
+      <name val="Arial"/>
       <family val="3"/>
       <sz val="12"/>
     </font>
     <font>
-      <name val="宋体"/>
-      <charset val="134"/>
+      <name val="Arial"/>
       <family val="3"/>
       <b val="1"/>
       <color indexed="56"/>
       <sz val="18"/>
     </font>
     <font>
-      <name val="宋体"/>
-      <charset val="134"/>
+      <name val="Arial"/>
       <family val="3"/>
       <b val="1"/>
       <color indexed="56"/>
       <sz val="15"/>
     </font>
     <font>
-      <name val="宋体"/>
-      <charset val="134"/>
+      <name val="Arial"/>
       <family val="3"/>
       <b val="1"/>
       <color indexed="56"/>
       <sz val="13"/>
     </font>
     <font>
-      <name val="宋体"/>
-      <charset val="134"/>
+      <name val="Arial"/>
       <family val="3"/>
       <b val="1"/>
       <color indexed="56"/>
       <sz val="11"/>
     </font>
     <font>
-      <name val="宋体"/>
-      <charset val="134"/>
+      <name val="Arial"/>
       <family val="3"/>
       <color indexed="20"/>
       <sz val="11"/>
     </font>
     <font>
-      <name val="宋体"/>
-      <charset val="134"/>
+      <name val="Arial"/>
       <family val="3"/>
       <color indexed="17"/>
       <sz val="11"/>
     </font>
     <font>
-      <name val="宋体"/>
-      <charset val="134"/>
+      <name val="Arial"/>
       <family val="3"/>
       <b val="1"/>
       <color indexed="8"/>
       <sz val="11"/>
     </font>
     <font>
-      <name val="宋体"/>
-      <charset val="134"/>
+      <name val="Arial"/>
       <family val="3"/>
       <b val="1"/>
       <color indexed="52"/>
       <sz val="11"/>
     </font>
     <font>
-      <name val="宋体"/>
-      <charset val="134"/>
+      <name val="Arial"/>
       <family val="3"/>
       <b val="1"/>
       <color indexed="9"/>
       <sz val="11"/>
     </font>
     <font>
-      <name val="宋体"/>
-      <charset val="134"/>
+      <name val="Arial"/>
       <family val="3"/>
       <i val="1"/>
       <color indexed="23"/>
       <sz val="11"/>
     </font>
     <font>
-      <name val="宋体"/>
-      <charset val="134"/>
+      <name val="Arial"/>
       <family val="3"/>
       <color indexed="10"/>
       <sz val="11"/>
     </font>
     <font>
-      <name val="宋体"/>
-      <charset val="134"/>
+      <name val="Arial"/>
       <family val="3"/>
       <color indexed="52"/>
       <sz val="11"/>
     </font>
     <font>
-      <name val="宋体"/>
-      <charset val="134"/>
+      <name val="Arial"/>
       <family val="3"/>
       <color indexed="60"/>
       <sz val="11"/>
     </font>
     <font>
-      <name val="宋体"/>
-      <charset val="134"/>
+      <name val="Arial"/>
       <family val="3"/>
       <b val="1"/>
       <color indexed="63"/>
       <sz val="11"/>
     </font>
     <font>
-      <name val="宋体"/>
-      <charset val="134"/>
+      <name val="Arial"/>
       <family val="3"/>
       <color indexed="62"/>
       <sz val="11"/>
     </font>
     <font>
-      <name val="宋体"/>
-      <charset val="134"/>
+      <name val="Arial"/>
       <family val="3"/>
       <sz val="9"/>
     </font>
@@ -176,53 +158,45 @@
       <sz val="12"/>
     </font>
     <font>
-      <name val="宋体"/>
-      <charset val="134"/>
+      <name val="Arial"/>
       <family val="3"/>
       <b val="1"/>
       <sz val="24"/>
     </font>
     <font>
-      <name val="宋体"/>
-      <charset val="134"/>
+      <name val="Arial"/>
       <family val="3"/>
       <sz val="12"/>
     </font>
     <font>
-      <name val="宋体"/>
-      <charset val="134"/>
+      <name val="Arial"/>
       <family val="3"/>
       <b val="1"/>
       <sz val="12"/>
     </font>
     <font>
-      <name val="华文行楷"/>
-      <charset val="134"/>
+      <name val="Arial"/>
       <family val="3"/>
       <sz val="18"/>
     </font>
     <font>
-      <name val="宋体"/>
-      <charset val="134"/>
+      <name val="Arial"/>
       <family val="3"/>
       <sz val="10"/>
     </font>
     <font>
-      <name val="宋体"/>
-      <charset val="134"/>
+      <name val="Arial"/>
       <family val="3"/>
       <b val="1"/>
       <sz val="10"/>
     </font>
     <font>
-      <name val="宋体"/>
-      <charset val="134"/>
+      <name val="Arial"/>
       <family val="3"/>
       <sz val="11"/>
     </font>
     <font>
-      <name val="宋体"/>
-      <charset val="134"/>
+      <name val="Arial"/>
       <family val="3"/>
       <sz val="12"/>
     </font>
@@ -589,7 +563,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="66">
+  <cellXfs count="72">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
@@ -765,6 +739,24 @@
     </xf>
     <xf numFmtId="164" fontId="30" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="28" fillId="0" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="28" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="18">
@@ -1231,128 +1223,128 @@
       <c r="S1" s="56" t="n"/>
     </row>
     <row r="2" ht="16" customHeight="1">
-      <c r="A2" s="57" t="inlineStr">
+      <c r="A2" s="66" t="inlineStr">
         <is>
           <t>Наименование изделия: XXX</t>
         </is>
       </c>
-      <c r="B2" s="58" t="n"/>
-      <c r="C2" s="58" t="n"/>
-      <c r="D2" s="58" t="inlineStr">
+      <c r="B2" s="67" t="n"/>
+      <c r="C2" s="67" t="n"/>
+      <c r="D2" s="67" t="inlineStr">
         <is>
           <t>Обозначение изделия: XXX</t>
         </is>
       </c>
-      <c r="E2" s="58" t="n"/>
-      <c r="F2" s="58" t="n"/>
-      <c r="G2" s="58" t="n"/>
-      <c r="H2" s="58" t="n"/>
-      <c r="I2" s="58" t="inlineStr">
+      <c r="E2" s="67" t="n"/>
+      <c r="F2" s="67" t="n"/>
+      <c r="G2" s="67" t="n"/>
+      <c r="H2" s="67" t="n"/>
+      <c r="I2" s="67" t="inlineStr">
         <is>
           <t>Составил:</t>
         </is>
       </c>
-      <c r="J2" s="58" t="inlineStr">
+      <c r="J2" s="67" t="inlineStr">
         <is>
           <t>Дата:</t>
         </is>
       </c>
-      <c r="K2" s="58" t="n"/>
-      <c r="L2" s="59" t="n"/>
-      <c r="M2" s="59" t="n"/>
-      <c r="N2" s="59" t="n"/>
-      <c r="O2" s="59" t="n"/>
+      <c r="K2" s="67" t="n"/>
+      <c r="L2" s="68" t="n"/>
+      <c r="M2" s="68" t="n"/>
+      <c r="N2" s="68" t="n"/>
+      <c r="O2" s="68" t="n"/>
       <c r="P2" s="56" t="n"/>
       <c r="Q2" s="56" t="n"/>
       <c r="R2" s="56" t="n"/>
       <c r="S2" s="56" t="n"/>
     </row>
     <row r="3" ht="16" customHeight="1">
-      <c r="A3" s="60" t="inlineStr">
+      <c r="A3" s="69" t="inlineStr">
         <is>
           <t>Модель изделия: XXX</t>
         </is>
       </c>
-      <c r="B3" s="61" t="n"/>
-      <c r="C3" s="61" t="n"/>
-      <c r="D3" s="61" t="inlineStr">
+      <c r="B3" s="70" t="n"/>
+      <c r="C3" s="70" t="n"/>
+      <c r="D3" s="70" t="inlineStr">
         <is>
           <t>Версия:</t>
         </is>
       </c>
-      <c r="E3" s="61" t="n"/>
-      <c r="F3" s="61" t="n"/>
-      <c r="G3" s="61" t="n"/>
-      <c r="H3" s="61" t="n"/>
-      <c r="I3" s="58" t="inlineStr">
+      <c r="E3" s="70" t="n"/>
+      <c r="F3" s="70" t="n"/>
+      <c r="G3" s="70" t="n"/>
+      <c r="H3" s="70" t="n"/>
+      <c r="I3" s="67" t="inlineStr">
         <is>
           <t>Проверил:</t>
         </is>
       </c>
-      <c r="J3" s="58" t="inlineStr">
+      <c r="J3" s="67" t="inlineStr">
         <is>
           <t>Дата:</t>
         </is>
       </c>
-      <c r="K3" s="58" t="n"/>
-      <c r="L3" s="59" t="n"/>
-      <c r="M3" s="59" t="n"/>
-      <c r="N3" s="59" t="n"/>
-      <c r="O3" s="59" t="n"/>
+      <c r="K3" s="67" t="n"/>
+      <c r="L3" s="68" t="n"/>
+      <c r="M3" s="68" t="n"/>
+      <c r="N3" s="68" t="n"/>
+      <c r="O3" s="68" t="n"/>
       <c r="P3" s="56" t="n"/>
       <c r="Q3" s="56" t="n"/>
       <c r="R3" s="56" t="n"/>
       <c r="S3" s="56" t="n"/>
     </row>
     <row r="4" ht="16" customHeight="1">
-      <c r="A4" s="59" t="n"/>
-      <c r="B4" s="59" t="n"/>
-      <c r="C4" s="59" t="n"/>
-      <c r="D4" s="59" t="n"/>
-      <c r="E4" s="59" t="n"/>
-      <c r="F4" s="59" t="n"/>
-      <c r="G4" s="59" t="n"/>
-      <c r="H4" s="59" t="n"/>
-      <c r="I4" s="58" t="inlineStr">
+      <c r="A4" s="68" t="n"/>
+      <c r="B4" s="68" t="n"/>
+      <c r="C4" s="68" t="n"/>
+      <c r="D4" s="68" t="n"/>
+      <c r="E4" s="68" t="n"/>
+      <c r="F4" s="68" t="n"/>
+      <c r="G4" s="68" t="n"/>
+      <c r="H4" s="68" t="n"/>
+      <c r="I4" s="67" t="inlineStr">
         <is>
           <t>Утвердил:</t>
         </is>
       </c>
-      <c r="J4" s="58" t="inlineStr">
+      <c r="J4" s="67" t="inlineStr">
         <is>
           <t>Дата:</t>
         </is>
       </c>
-      <c r="K4" s="58" t="n"/>
-      <c r="L4" s="59" t="n"/>
-      <c r="M4" s="59" t="n"/>
-      <c r="N4" s="59" t="n"/>
-      <c r="O4" s="59" t="n"/>
+      <c r="K4" s="67" t="n"/>
+      <c r="L4" s="68" t="n"/>
+      <c r="M4" s="68" t="n"/>
+      <c r="N4" s="68" t="n"/>
+      <c r="O4" s="68" t="n"/>
       <c r="P4" s="56" t="n"/>
       <c r="Q4" s="56" t="n"/>
       <c r="R4" s="56" t="n"/>
       <c r="S4" s="56" t="n"/>
     </row>
     <row r="5" ht="16" customHeight="1">
-      <c r="A5" s="58" t="n"/>
-      <c r="B5" s="58" t="n"/>
-      <c r="C5" s="58" t="n"/>
-      <c r="D5" s="58" t="n"/>
-      <c r="E5" s="58" t="n"/>
-      <c r="F5" s="58" t="n"/>
-      <c r="G5" s="58" t="n"/>
-      <c r="H5" s="58" t="n"/>
-      <c r="I5" s="58" t="inlineStr">
+      <c r="A5" s="67" t="n"/>
+      <c r="B5" s="67" t="n"/>
+      <c r="C5" s="67" t="n"/>
+      <c r="D5" s="67" t="n"/>
+      <c r="E5" s="67" t="n"/>
+      <c r="F5" s="67" t="n"/>
+      <c r="G5" s="67" t="n"/>
+      <c r="H5" s="67" t="n"/>
+      <c r="I5" s="67" t="inlineStr">
         <is>
           <t>Номер таблицы:</t>
         </is>
       </c>
-      <c r="J5" s="58" t="n"/>
-      <c r="K5" s="58" t="n"/>
-      <c r="L5" s="59" t="n"/>
-      <c r="M5" s="59" t="n"/>
-      <c r="N5" s="59" t="n"/>
-      <c r="O5" s="59" t="n"/>
+      <c r="J5" s="67" t="n"/>
+      <c r="K5" s="67" t="n"/>
+      <c r="L5" s="68" t="n"/>
+      <c r="M5" s="68" t="n"/>
+      <c r="N5" s="68" t="n"/>
+      <c r="O5" s="68" t="n"/>
       <c r="P5" s="56" t="n"/>
       <c r="Q5" s="56" t="n"/>
       <c r="R5" s="56" t="n"/>
@@ -1456,7 +1448,7 @@
       <c r="L7" s="45" t="n"/>
       <c r="M7" s="45" t="n"/>
       <c r="N7" s="45" t="n"/>
-      <c r="O7" s="62" t="n"/>
+      <c r="O7" s="71" t="n"/>
       <c r="P7" s="56" t="n"/>
       <c r="Q7" s="56" t="n"/>
       <c r="R7" s="56" t="n"/>
@@ -1477,7 +1469,7 @@
       <c r="L8" s="45" t="n"/>
       <c r="M8" s="45" t="n"/>
       <c r="N8" s="45" t="n"/>
-      <c r="O8" s="62" t="n"/>
+      <c r="O8" s="71" t="n"/>
       <c r="P8" s="56" t="n"/>
       <c r="Q8" s="56" t="n"/>
       <c r="R8" s="56" t="n"/>
@@ -1498,7 +1490,7 @@
       <c r="L9" s="45" t="n"/>
       <c r="M9" s="45" t="n"/>
       <c r="N9" s="45" t="n"/>
-      <c r="O9" s="62" t="n"/>
+      <c r="O9" s="71" t="n"/>
       <c r="P9" s="56" t="n"/>
       <c r="Q9" s="56" t="n"/>
       <c r="R9" s="56" t="n"/>
@@ -1519,7 +1511,7 @@
       <c r="L10" s="45" t="n"/>
       <c r="M10" s="45" t="n"/>
       <c r="N10" s="45" t="n"/>
-      <c r="O10" s="62" t="n"/>
+      <c r="O10" s="71" t="n"/>
       <c r="P10" s="56" t="n"/>
       <c r="Q10" s="56" t="n"/>
       <c r="R10" s="56" t="n"/>
@@ -1540,7 +1532,7 @@
       <c r="L11" s="45" t="n"/>
       <c r="M11" s="45" t="n"/>
       <c r="N11" s="45" t="n"/>
-      <c r="O11" s="62" t="n"/>
+      <c r="O11" s="71" t="n"/>
       <c r="P11" s="56" t="n"/>
       <c r="Q11" s="56" t="n"/>
       <c r="R11" s="56" t="n"/>
@@ -1561,7 +1553,7 @@
       <c r="L12" s="45" t="n"/>
       <c r="M12" s="45" t="n"/>
       <c r="N12" s="45" t="n"/>
-      <c r="O12" s="62" t="n"/>
+      <c r="O12" s="71" t="n"/>
       <c r="P12" s="56" t="n"/>
       <c r="Q12" s="56" t="n"/>
       <c r="R12" s="56" t="n"/>
@@ -1582,7 +1574,7 @@
       <c r="L13" s="45" t="n"/>
       <c r="M13" s="45" t="n"/>
       <c r="N13" s="45" t="n"/>
-      <c r="O13" s="62" t="n"/>
+      <c r="O13" s="71" t="n"/>
       <c r="P13" s="56" t="n"/>
       <c r="Q13" s="56" t="n"/>
       <c r="R13" s="56" t="n"/>
@@ -1603,7 +1595,7 @@
       <c r="L14" s="45" t="n"/>
       <c r="M14" s="45" t="n"/>
       <c r="N14" s="45" t="n"/>
-      <c r="O14" s="62" t="n"/>
+      <c r="O14" s="71" t="n"/>
       <c r="P14" s="56" t="n"/>
       <c r="Q14" s="56" t="n"/>
       <c r="R14" s="56" t="n"/>
@@ -1624,7 +1616,7 @@
       <c r="L15" s="45" t="n"/>
       <c r="M15" s="45" t="n"/>
       <c r="N15" s="45" t="n"/>
-      <c r="O15" s="62" t="n"/>
+      <c r="O15" s="71" t="n"/>
       <c r="P15" s="56" t="n"/>
       <c r="Q15" s="56" t="n"/>
       <c r="R15" s="56" t="n"/>
@@ -1645,7 +1637,7 @@
       <c r="L16" s="45" t="n"/>
       <c r="M16" s="45" t="n"/>
       <c r="N16" s="45" t="n"/>
-      <c r="O16" s="62" t="n"/>
+      <c r="O16" s="71" t="n"/>
       <c r="P16" s="56" t="n"/>
       <c r="Q16" s="56" t="n"/>
       <c r="R16" s="56" t="n"/>
@@ -1666,7 +1658,7 @@
       <c r="L17" s="45" t="n"/>
       <c r="M17" s="45" t="n"/>
       <c r="N17" s="45" t="n"/>
-      <c r="O17" s="62" t="n"/>
+      <c r="O17" s="71" t="n"/>
       <c r="P17" s="56" t="n"/>
       <c r="Q17" s="56" t="n"/>
       <c r="R17" s="56" t="n"/>
@@ -1687,7 +1679,7 @@
       <c r="L18" s="45" t="n"/>
       <c r="M18" s="45" t="n"/>
       <c r="N18" s="45" t="n"/>
-      <c r="O18" s="62" t="n"/>
+      <c r="O18" s="71" t="n"/>
       <c r="P18" s="56" t="n"/>
       <c r="Q18" s="56" t="n"/>
       <c r="R18" s="56" t="n"/>
@@ -1708,7 +1700,7 @@
       <c r="L19" s="45" t="n"/>
       <c r="M19" s="45" t="n"/>
       <c r="N19" s="45" t="n"/>
-      <c r="O19" s="62" t="n"/>
+      <c r="O19" s="71" t="n"/>
       <c r="P19" s="56" t="n"/>
       <c r="Q19" s="56" t="n"/>
       <c r="R19" s="56" t="n"/>
@@ -1729,7 +1721,7 @@
       <c r="L20" s="45" t="n"/>
       <c r="M20" s="45" t="n"/>
       <c r="N20" s="45" t="n"/>
-      <c r="O20" s="62" t="n"/>
+      <c r="O20" s="71" t="n"/>
       <c r="P20" s="56" t="n"/>
       <c r="Q20" s="56" t="n"/>
       <c r="R20" s="56" t="n"/>
@@ -1750,7 +1742,7 @@
       <c r="L21" s="45" t="n"/>
       <c r="M21" s="45" t="n"/>
       <c r="N21" s="45" t="n"/>
-      <c r="O21" s="62" t="n"/>
+      <c r="O21" s="71" t="n"/>
       <c r="P21" s="56" t="n"/>
       <c r="Q21" s="56" t="n"/>
       <c r="R21" s="56" t="n"/>
@@ -1771,7 +1763,7 @@
       <c r="L22" s="45" t="n"/>
       <c r="M22" s="45" t="n"/>
       <c r="N22" s="45" t="n"/>
-      <c r="O22" s="62" t="n"/>
+      <c r="O22" s="71" t="n"/>
       <c r="P22" s="56" t="n"/>
       <c r="Q22" s="56" t="n"/>
       <c r="R22" s="56" t="n"/>
@@ -1792,7 +1784,7 @@
       <c r="L23" s="45" t="n"/>
       <c r="M23" s="45" t="n"/>
       <c r="N23" s="45" t="n"/>
-      <c r="O23" s="62" t="n"/>
+      <c r="O23" s="71" t="n"/>
       <c r="P23" s="56" t="n"/>
       <c r="Q23" s="56" t="n"/>
       <c r="R23" s="56" t="n"/>
@@ -1813,7 +1805,7 @@
       <c r="L24" s="45" t="n"/>
       <c r="M24" s="45" t="n"/>
       <c r="N24" s="45" t="n"/>
-      <c r="O24" s="62" t="n"/>
+      <c r="O24" s="71" t="n"/>
       <c r="P24" s="56" t="n"/>
       <c r="Q24" s="56" t="n"/>
       <c r="R24" s="56" t="n"/>
@@ -1834,7 +1826,7 @@
       <c r="L25" s="45" t="n"/>
       <c r="M25" s="45" t="n"/>
       <c r="N25" s="45" t="n"/>
-      <c r="O25" s="62" t="n"/>
+      <c r="O25" s="71" t="n"/>
       <c r="P25" s="56" t="n"/>
       <c r="Q25" s="56" t="n"/>
       <c r="R25" s="56" t="n"/>
@@ -1855,7 +1847,7 @@
       <c r="L26" s="45" t="n"/>
       <c r="M26" s="45" t="n"/>
       <c r="N26" s="45" t="n"/>
-      <c r="O26" s="62" t="n"/>
+      <c r="O26" s="71" t="n"/>
       <c r="P26" s="56" t="n"/>
       <c r="Q26" s="56" t="n"/>
       <c r="R26" s="56" t="n"/>
@@ -1876,7 +1868,7 @@
       <c r="L27" s="45" t="n"/>
       <c r="M27" s="45" t="n"/>
       <c r="N27" s="45" t="n"/>
-      <c r="O27" s="62" t="n"/>
+      <c r="O27" s="71" t="n"/>
       <c r="P27" s="56" t="n"/>
       <c r="Q27" s="56" t="n"/>
       <c r="R27" s="56" t="n"/>
@@ -1897,7 +1889,7 @@
       <c r="L28" s="45" t="n"/>
       <c r="M28" s="45" t="n"/>
       <c r="N28" s="45" t="n"/>
-      <c r="O28" s="62" t="n"/>
+      <c r="O28" s="71" t="n"/>
       <c r="P28" s="56" t="n"/>
       <c r="Q28" s="56" t="n"/>
       <c r="R28" s="56" t="n"/>
@@ -1918,7 +1910,7 @@
       <c r="L29" s="45" t="n"/>
       <c r="M29" s="45" t="n"/>
       <c r="N29" s="45" t="n"/>
-      <c r="O29" s="62" t="n"/>
+      <c r="O29" s="71" t="n"/>
       <c r="P29" s="56" t="n"/>
       <c r="Q29" s="56" t="n"/>
       <c r="R29" s="56" t="n"/>
@@ -1939,7 +1931,7 @@
       <c r="L30" s="45" t="n"/>
       <c r="M30" s="45" t="n"/>
       <c r="N30" s="45" t="n"/>
-      <c r="O30" s="62" t="n"/>
+      <c r="O30" s="71" t="n"/>
       <c r="P30" s="56" t="n"/>
       <c r="Q30" s="56" t="n"/>
       <c r="R30" s="56" t="n"/>
@@ -1960,7 +1952,7 @@
       <c r="L31" s="45" t="n"/>
       <c r="M31" s="45" t="n"/>
       <c r="N31" s="45" t="n"/>
-      <c r="O31" s="62" t="n"/>
+      <c r="O31" s="71" t="n"/>
       <c r="P31" s="56" t="n"/>
       <c r="Q31" s="56" t="n"/>
       <c r="R31" s="56" t="n"/>
@@ -1981,7 +1973,7 @@
       <c r="L32" s="45" t="n"/>
       <c r="M32" s="45" t="n"/>
       <c r="N32" s="45" t="n"/>
-      <c r="O32" s="62" t="n"/>
+      <c r="O32" s="71" t="n"/>
       <c r="P32" s="56" t="n"/>
       <c r="Q32" s="56" t="n"/>
       <c r="R32" s="56" t="n"/>
@@ -2002,7 +1994,7 @@
       <c r="L33" s="45" t="n"/>
       <c r="M33" s="45" t="n"/>
       <c r="N33" s="45" t="n"/>
-      <c r="O33" s="62" t="n"/>
+      <c r="O33" s="71" t="n"/>
       <c r="P33" s="56" t="n"/>
       <c r="Q33" s="56" t="n"/>
       <c r="R33" s="56" t="n"/>
@@ -2023,7 +2015,7 @@
       <c r="L34" s="45" t="n"/>
       <c r="M34" s="45" t="n"/>
       <c r="N34" s="45" t="n"/>
-      <c r="O34" s="62" t="n"/>
+      <c r="O34" s="71" t="n"/>
       <c r="P34" s="56" t="n"/>
       <c r="Q34" s="56" t="n"/>
       <c r="R34" s="56" t="n"/>
@@ -2044,7 +2036,7 @@
       <c r="L35" s="45" t="n"/>
       <c r="M35" s="45" t="n"/>
       <c r="N35" s="45" t="n"/>
-      <c r="O35" s="62" t="n"/>
+      <c r="O35" s="71" t="n"/>
       <c r="P35" s="56" t="n"/>
       <c r="Q35" s="56" t="n"/>
       <c r="R35" s="56" t="n"/>
@@ -2065,7 +2057,7 @@
       <c r="L36" s="45" t="n"/>
       <c r="M36" s="45" t="n"/>
       <c r="N36" s="45" t="n"/>
-      <c r="O36" s="62" t="n"/>
+      <c r="O36" s="71" t="n"/>
       <c r="P36" s="56" t="n"/>
       <c r="Q36" s="56" t="n"/>
       <c r="R36" s="56" t="n"/>
@@ -2086,7 +2078,7 @@
       <c r="L37" s="45" t="n"/>
       <c r="M37" s="45" t="n"/>
       <c r="N37" s="45" t="n"/>
-      <c r="O37" s="62" t="n"/>
+      <c r="O37" s="71" t="n"/>
       <c r="P37" s="56" t="n"/>
       <c r="Q37" s="56" t="n"/>
       <c r="R37" s="56" t="n"/>
@@ -2107,7 +2099,7 @@
       <c r="L38" s="45" t="n"/>
       <c r="M38" s="45" t="n"/>
       <c r="N38" s="45" t="n"/>
-      <c r="O38" s="62" t="n"/>
+      <c r="O38" s="71" t="n"/>
       <c r="P38" s="56" t="n"/>
       <c r="Q38" s="56" t="n"/>
       <c r="R38" s="56" t="n"/>
@@ -2128,7 +2120,7 @@
       <c r="L39" s="45" t="n"/>
       <c r="M39" s="45" t="n"/>
       <c r="N39" s="45" t="n"/>
-      <c r="O39" s="62" t="n"/>
+      <c r="O39" s="71" t="n"/>
       <c r="P39" s="56" t="n"/>
       <c r="Q39" s="56" t="n"/>
       <c r="R39" s="56" t="n"/>
@@ -2149,7 +2141,7 @@
       <c r="L40" s="45" t="n"/>
       <c r="M40" s="45" t="n"/>
       <c r="N40" s="45" t="n"/>
-      <c r="O40" s="62" t="n"/>
+      <c r="O40" s="71" t="n"/>
       <c r="P40" s="56" t="n"/>
       <c r="Q40" s="56" t="n"/>
       <c r="R40" s="56" t="n"/>
@@ -2170,7 +2162,7 @@
       <c r="L41" s="45" t="n"/>
       <c r="M41" s="45" t="n"/>
       <c r="N41" s="45" t="n"/>
-      <c r="O41" s="62" t="n"/>
+      <c r="O41" s="71" t="n"/>
       <c r="P41" s="56" t="n"/>
       <c r="Q41" s="56" t="n"/>
       <c r="R41" s="56" t="n"/>
@@ -2191,7 +2183,7 @@
       <c r="L42" s="45" t="n"/>
       <c r="M42" s="45" t="n"/>
       <c r="N42" s="45" t="n"/>
-      <c r="O42" s="62" t="n"/>
+      <c r="O42" s="71" t="n"/>
       <c r="P42" s="56" t="n"/>
       <c r="Q42" s="56" t="n"/>
       <c r="R42" s="56" t="n"/>
@@ -2212,7 +2204,7 @@
       <c r="L43" s="45" t="n"/>
       <c r="M43" s="45" t="n"/>
       <c r="N43" s="45" t="n"/>
-      <c r="O43" s="62" t="n"/>
+      <c r="O43" s="71" t="n"/>
       <c r="P43" s="56" t="n"/>
       <c r="Q43" s="56" t="n"/>
       <c r="R43" s="56" t="n"/>
@@ -2233,7 +2225,7 @@
       <c r="L44" s="45" t="n"/>
       <c r="M44" s="45" t="n"/>
       <c r="N44" s="45" t="n"/>
-      <c r="O44" s="62" t="n"/>
+      <c r="O44" s="71" t="n"/>
       <c r="P44" s="56" t="n"/>
       <c r="Q44" s="56" t="n"/>
       <c r="R44" s="56" t="n"/>
@@ -2254,7 +2246,7 @@
       <c r="L45" s="45" t="n"/>
       <c r="M45" s="45" t="n"/>
       <c r="N45" s="45" t="n"/>
-      <c r="O45" s="62" t="n"/>
+      <c r="O45" s="71" t="n"/>
       <c r="P45" s="56" t="n"/>
       <c r="Q45" s="56" t="n"/>
       <c r="R45" s="56" t="n"/>
@@ -2275,7 +2267,7 @@
       <c r="L46" s="45" t="n"/>
       <c r="M46" s="45" t="n"/>
       <c r="N46" s="45" t="n"/>
-      <c r="O46" s="62" t="n"/>
+      <c r="O46" s="71" t="n"/>
       <c r="P46" s="63" t="n"/>
       <c r="Q46" s="63" t="n"/>
       <c r="R46" s="64" t="n"/>
@@ -2296,7 +2288,7 @@
       <c r="L47" s="45" t="n"/>
       <c r="M47" s="45" t="n"/>
       <c r="N47" s="45" t="n"/>
-      <c r="O47" s="62" t="n"/>
+      <c r="O47" s="71" t="n"/>
       <c r="P47" s="56" t="n"/>
       <c r="Q47" s="56" t="n"/>
       <c r="R47" s="56" t="n"/>
@@ -2317,7 +2309,7 @@
       <c r="L48" s="45" t="n"/>
       <c r="M48" s="45" t="n"/>
       <c r="N48" s="45" t="n"/>
-      <c r="O48" s="62" t="n"/>
+      <c r="O48" s="71" t="n"/>
       <c r="P48" s="56" t="n"/>
       <c r="Q48" s="56" t="n"/>
       <c r="R48" s="56" t="n"/>
@@ -2338,7 +2330,7 @@
       <c r="L49" s="45" t="n"/>
       <c r="M49" s="45" t="n"/>
       <c r="N49" s="45" t="n"/>
-      <c r="O49" s="62" t="n"/>
+      <c r="O49" s="71" t="n"/>
       <c r="P49" s="56" t="n"/>
       <c r="Q49" s="56" t="n"/>
       <c r="R49" s="56" t="n"/>
@@ -2359,7 +2351,7 @@
       <c r="L50" s="45" t="n"/>
       <c r="M50" s="45" t="n"/>
       <c r="N50" s="45" t="n"/>
-      <c r="O50" s="62" t="n"/>
+      <c r="O50" s="71" t="n"/>
       <c r="P50" s="56" t="n"/>
       <c r="Q50" s="56" t="n"/>
       <c r="R50" s="56" t="n"/>
@@ -2380,7 +2372,7 @@
       <c r="L51" s="45" t="n"/>
       <c r="M51" s="45" t="n"/>
       <c r="N51" s="45" t="n"/>
-      <c r="O51" s="62" t="n"/>
+      <c r="O51" s="71" t="n"/>
       <c r="P51" s="56" t="n"/>
       <c r="Q51" s="56" t="n"/>
       <c r="R51" s="56" t="n"/>
@@ -2401,7 +2393,7 @@
       <c r="L52" s="45" t="n"/>
       <c r="M52" s="45" t="n"/>
       <c r="N52" s="45" t="n"/>
-      <c r="O52" s="62" t="n"/>
+      <c r="O52" s="71" t="n"/>
       <c r="P52" s="56" t="n"/>
       <c r="Q52" s="56" t="n"/>
       <c r="R52" s="56" t="n"/>
@@ -2422,7 +2414,7 @@
       <c r="L53" s="45" t="n"/>
       <c r="M53" s="45" t="n"/>
       <c r="N53" s="45" t="n"/>
-      <c r="O53" s="62" t="n"/>
+      <c r="O53" s="71" t="n"/>
       <c r="P53" s="56" t="n"/>
       <c r="Q53" s="56" t="n"/>
       <c r="R53" s="56" t="n"/>
@@ -2443,7 +2435,7 @@
       <c r="L54" s="45" t="n"/>
       <c r="M54" s="45" t="n"/>
       <c r="N54" s="45" t="n"/>
-      <c r="O54" s="62" t="n"/>
+      <c r="O54" s="71" t="n"/>
       <c r="P54" s="63" t="n"/>
       <c r="Q54" s="63" t="n"/>
       <c r="R54" s="64" t="n"/>
@@ -2464,7 +2456,7 @@
       <c r="L55" s="45" t="n"/>
       <c r="M55" s="45" t="n"/>
       <c r="N55" s="45" t="n"/>
-      <c r="O55" s="62" t="n"/>
+      <c r="O55" s="71" t="n"/>
       <c r="P55" s="56" t="n"/>
       <c r="Q55" s="56" t="n"/>
       <c r="R55" s="56" t="n"/>
@@ -2485,7 +2477,7 @@
       <c r="L56" s="45" t="n"/>
       <c r="M56" s="45" t="n"/>
       <c r="N56" s="45" t="n"/>
-      <c r="O56" s="62" t="n"/>
+      <c r="O56" s="71" t="n"/>
       <c r="P56" s="56" t="n"/>
       <c r="Q56" s="56" t="n"/>
       <c r="R56" s="56" t="n"/>
@@ -2506,7 +2498,7 @@
       <c r="L57" s="45" t="n"/>
       <c r="M57" s="45" t="n"/>
       <c r="N57" s="45" t="n"/>
-      <c r="O57" s="62" t="n"/>
+      <c r="O57" s="71" t="n"/>
       <c r="P57" s="56" t="n"/>
       <c r="Q57" s="56" t="n"/>
       <c r="R57" s="56" t="n"/>
@@ -2527,7 +2519,7 @@
       <c r="L58" s="45" t="n"/>
       <c r="M58" s="45" t="n"/>
       <c r="N58" s="45" t="n"/>
-      <c r="O58" s="62" t="n"/>
+      <c r="O58" s="71" t="n"/>
       <c r="P58" s="63" t="n"/>
       <c r="Q58" s="63" t="n"/>
       <c r="R58" s="64" t="n"/>
@@ -2548,7 +2540,7 @@
       <c r="L59" s="45" t="n"/>
       <c r="M59" s="45" t="n"/>
       <c r="N59" s="45" t="n"/>
-      <c r="O59" s="62" t="n"/>
+      <c r="O59" s="71" t="n"/>
       <c r="P59" s="56" t="n"/>
       <c r="Q59" s="56" t="n"/>
       <c r="R59" s="56" t="n"/>
@@ -2569,7 +2561,7 @@
       <c r="L60" s="45" t="n"/>
       <c r="M60" s="45" t="n"/>
       <c r="N60" s="45" t="n"/>
-      <c r="O60" s="62" t="n"/>
+      <c r="O60" s="71" t="n"/>
       <c r="P60" s="56" t="n"/>
       <c r="Q60" s="56" t="n"/>
       <c r="R60" s="56" t="n"/>
@@ -2590,7 +2582,7 @@
       <c r="L61" s="45" t="n"/>
       <c r="M61" s="45" t="n"/>
       <c r="N61" s="45" t="n"/>
-      <c r="O61" s="62" t="n"/>
+      <c r="O61" s="71" t="n"/>
       <c r="P61" s="56" t="n"/>
       <c r="Q61" s="56" t="n"/>
       <c r="R61" s="56" t="n"/>
@@ -2611,7 +2603,7 @@
       <c r="L62" s="45" t="n"/>
       <c r="M62" s="45" t="n"/>
       <c r="N62" s="45" t="n"/>
-      <c r="O62" s="62" t="n"/>
+      <c r="O62" s="71" t="n"/>
       <c r="P62" s="56" t="n"/>
       <c r="Q62" s="56" t="n"/>
       <c r="R62" s="56" t="n"/>
@@ -2632,7 +2624,7 @@
       <c r="L63" s="45" t="n"/>
       <c r="M63" s="45" t="n"/>
       <c r="N63" s="45" t="n"/>
-      <c r="O63" s="62" t="n"/>
+      <c r="O63" s="71" t="n"/>
       <c r="P63" s="56" t="n"/>
       <c r="Q63" s="56" t="n"/>
       <c r="R63" s="56" t="n"/>
@@ -2653,7 +2645,7 @@
       <c r="L64" s="45" t="n"/>
       <c r="M64" s="45" t="n"/>
       <c r="N64" s="45" t="n"/>
-      <c r="O64" s="62" t="n"/>
+      <c r="O64" s="71" t="n"/>
       <c r="P64" s="56" t="n"/>
       <c r="Q64" s="56" t="n"/>
       <c r="R64" s="56" t="n"/>
@@ -2674,7 +2666,7 @@
       <c r="L65" s="45" t="n"/>
       <c r="M65" s="45" t="n"/>
       <c r="N65" s="45" t="n"/>
-      <c r="O65" s="62" t="n"/>
+      <c r="O65" s="71" t="n"/>
       <c r="P65" s="56" t="n"/>
       <c r="Q65" s="56" t="n"/>
       <c r="R65" s="56" t="n"/>
@@ -2695,7 +2687,7 @@
       <c r="L66" s="45" t="n"/>
       <c r="M66" s="45" t="n"/>
       <c r="N66" s="45" t="n"/>
-      <c r="O66" s="62" t="n"/>
+      <c r="O66" s="71" t="n"/>
       <c r="P66" s="56" t="n"/>
       <c r="Q66" s="56" t="n"/>
       <c r="R66" s="56" t="n"/>
@@ -2716,7 +2708,7 @@
       <c r="L67" s="45" t="n"/>
       <c r="M67" s="45" t="n"/>
       <c r="N67" s="45" t="n"/>
-      <c r="O67" s="62" t="n"/>
+      <c r="O67" s="71" t="n"/>
       <c r="P67" s="56" t="n"/>
       <c r="Q67" s="56" t="n"/>
       <c r="R67" s="56" t="n"/>
@@ -2737,7 +2729,7 @@
       <c r="L68" s="45" t="n"/>
       <c r="M68" s="45" t="n"/>
       <c r="N68" s="45" t="n"/>
-      <c r="O68" s="62" t="n"/>
+      <c r="O68" s="71" t="n"/>
       <c r="P68" s="56" t="n"/>
       <c r="Q68" s="56" t="n"/>
       <c r="R68" s="56" t="n"/>
@@ -2758,7 +2750,7 @@
       <c r="L69" s="45" t="n"/>
       <c r="M69" s="45" t="n"/>
       <c r="N69" s="45" t="n"/>
-      <c r="O69" s="62" t="n"/>
+      <c r="O69" s="71" t="n"/>
       <c r="P69" s="56" t="n"/>
       <c r="Q69" s="56" t="n"/>
       <c r="R69" s="56" t="n"/>
@@ -2779,7 +2771,7 @@
       <c r="L70" s="45" t="n"/>
       <c r="M70" s="45" t="n"/>
       <c r="N70" s="45" t="n"/>
-      <c r="O70" s="62" t="n"/>
+      <c r="O70" s="71" t="n"/>
       <c r="P70" s="56" t="n"/>
       <c r="Q70" s="56" t="n"/>
       <c r="R70" s="56" t="n"/>
@@ -2800,7 +2792,7 @@
       <c r="L71" s="45" t="n"/>
       <c r="M71" s="45" t="n"/>
       <c r="N71" s="45" t="n"/>
-      <c r="O71" s="62" t="n"/>
+      <c r="O71" s="71" t="n"/>
       <c r="P71" s="56" t="n"/>
       <c r="Q71" s="56" t="n"/>
       <c r="R71" s="56" t="n"/>
@@ -2821,7 +2813,7 @@
       <c r="L72" s="45" t="n"/>
       <c r="M72" s="45" t="n"/>
       <c r="N72" s="45" t="n"/>
-      <c r="O72" s="62" t="n"/>
+      <c r="O72" s="71" t="n"/>
       <c r="P72" s="56" t="n"/>
       <c r="Q72" s="56" t="n"/>
       <c r="R72" s="56" t="n"/>
@@ -2842,7 +2834,7 @@
       <c r="L73" s="45" t="n"/>
       <c r="M73" s="45" t="n"/>
       <c r="N73" s="45" t="n"/>
-      <c r="O73" s="62" t="n"/>
+      <c r="O73" s="71" t="n"/>
       <c r="P73" s="56" t="n"/>
       <c r="Q73" s="56" t="n"/>
       <c r="R73" s="56" t="n"/>
@@ -2863,7 +2855,7 @@
       <c r="L74" s="45" t="n"/>
       <c r="M74" s="45" t="n"/>
       <c r="N74" s="45" t="n"/>
-      <c r="O74" s="62" t="n"/>
+      <c r="O74" s="71" t="n"/>
       <c r="P74" s="56" t="n"/>
       <c r="Q74" s="56" t="n"/>
       <c r="R74" s="56" t="n"/>
@@ -2884,7 +2876,7 @@
       <c r="L75" s="45" t="n"/>
       <c r="M75" s="45" t="n"/>
       <c r="N75" s="45" t="n"/>
-      <c r="O75" s="62" t="n"/>
+      <c r="O75" s="71" t="n"/>
       <c r="P75" s="56" t="n"/>
       <c r="Q75" s="56" t="n"/>
       <c r="R75" s="56" t="n"/>

</xml_diff>

<commit_message>
BOM: full Chinese->Russian removal, Frmmapping/anchor + binder fixes
- Template (bom_шаблон.xlsx): drop all Chinese defined names, keep a single
  fully-Russian set anchoring the same export cells (russify_bom_defined_names.py).
- SWTools.settings: namemappinglist mappingname values -> Russian; strip legacy
  Chinese tokens (机加/外购) from $Тип$ filter rules, keeping Russian values.
- Localizer: widen Frmmapping to every calculated/service Col_* column (except
  the non-data checkbox/new-folder columns); pin Frmsetpropname 'Импорт...'
  button to Bottom|Left so it stops drifting when the dialog is resized.
- VTBinder: resolve embedded assembly identities in nested type names via the
  Type.GetType resolver overload (fixes 'System.Object из ZTool' on Import);
  resolver methods kept as instance methods to avoid a cached-delegate helper
  type that would leave a dangling donor-assembly reference.
</commit_message>
<xml_diff>
--- a/Шаблоны спецификации/bom_шаблон.xlsx
+++ b/Шаблоны спецификации/bom_шаблон.xlsx
@@ -9,25 +9,20 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Спецификация" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="版本">Спецификация!$E$6</definedName>
-    <definedName name="表面处理">Спецификация!$I$6</definedName>
-    <definedName name="材质">Спецификация!$N$6</definedName>
-    <definedName name="磁盘文件名">Спецификация!$L$6</definedName>
-    <definedName name="类型">Спецификация!$H$6</definedName>
-    <definedName name="零件名称">Спецификация!$C$6</definedName>
-    <definedName name="路径">Спецификация!$O$6</definedName>
-    <definedName name="缩略图">Спецификация!$M$6</definedName>
-    <definedName name="统计数量">Спецификация!$G$6</definedName>
-    <definedName name="图号">Спецификация!$D$6</definedName>
-    <definedName name="序号">Спецификация!$A$6</definedName>
-    <definedName name="重量">Спецификация!$J$6</definedName>
     <definedName name="Номер">'Спецификация'!$A$6</definedName>
+    <definedName name="Наименование">'Спецификация'!$C$6</definedName>
+    <definedName name="Обозначение">'Спецификация'!$D$6</definedName>
+    <definedName name="Версия">'Спецификация'!$E$6</definedName>
+    <definedName name="ЕдИзм">'Спецификация'!$F$6</definedName>
     <definedName name="Количество">'Спецификация'!$G$6</definedName>
+    <definedName name="Тип">'Спецификация'!$H$6</definedName>
+    <definedName name="ОбработкаПоверхности">'Спецификация'!$I$6</definedName>
+    <definedName name="МассаЕдКг">'Спецификация'!$J$6</definedName>
+    <definedName name="ИмяФайла">'Спецификация'!$L$6</definedName>
+    <definedName name="Эскиз">'Спецификация'!$M$6</definedName>
+    <definedName name="Материал">'Спецификация'!$N$6</definedName>
     <definedName name="Путь">'Спецификация'!$O$6</definedName>
-    <definedName name="Эскиз">'Спецификация'!$M$6</definedName>
-    <definedName name="МассаЕдКг">'Спецификация'!$J$6</definedName>
     <definedName name="ГабаритныеРазмеры">'Спецификация'!$P$6</definedName>
-    <definedName name="ЕдИзм">'Спецификация'!$F$6</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Спецификация'!$1:$6</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'Спецификация'!$A$1:$P$75</definedName>
   </definedNames>

</xml_diff>

<commit_message>
fix: rename calculated BOM columns
</commit_message>
<xml_diff>
--- a/Шаблоны спецификации/bom_шаблон.xlsx
+++ b/Шаблоны спецификации/bom_шаблон.xlsx
@@ -310,7 +310,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="17">
+  <borders count="24">
     <border>
       <left/>
       <right/>
@@ -501,6 +501,55 @@
       <top style="thin"/>
       <bottom style="thin"/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right/>
+      <top/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -556,7 +605,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="59">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
@@ -703,6 +752,15 @@
     <xf numFmtId="14" fontId="30" fillId="0" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="18">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -1149,16 +1207,6 @@
           <t>Спецификация</t>
         </is>
       </c>
-      <c r="B1" s="34" t="n"/>
-      <c r="C1" s="34" t="n"/>
-      <c r="D1" s="34" t="n"/>
-      <c r="E1" s="34" t="n"/>
-      <c r="F1" s="34" t="n"/>
-      <c r="G1" s="34" t="n"/>
-      <c r="H1" s="34" t="n"/>
-      <c r="I1" s="34" t="n"/>
-      <c r="J1" s="34" t="n"/>
-      <c r="K1" s="34" t="n"/>
       <c r="L1" s="34" t="n"/>
       <c r="M1" s="34" t="n"/>
       <c r="N1" s="34" t="n"/>
@@ -1174,17 +1222,17 @@
           <t>Наименование изделия: XXX</t>
         </is>
       </c>
-      <c r="B2" s="37" t="n"/>
-      <c r="C2" s="37" t="n"/>
+      <c r="B2" s="50" t="n"/>
+      <c r="C2" s="50" t="n"/>
       <c r="D2" s="37" t="inlineStr">
         <is>
           <t>Обозначение изделия: XXX</t>
         </is>
       </c>
-      <c r="E2" s="37" t="n"/>
-      <c r="F2" s="37" t="n"/>
-      <c r="G2" s="37" t="n"/>
-      <c r="H2" s="37" t="n"/>
+      <c r="E2" s="50" t="n"/>
+      <c r="F2" s="50" t="n"/>
+      <c r="G2" s="50" t="n"/>
+      <c r="H2" s="50" t="n"/>
       <c r="I2" s="37" t="inlineStr">
         <is>
           <t>Составил:</t>
@@ -1195,7 +1243,7 @@
           <t>Дата:</t>
         </is>
       </c>
-      <c r="K2" s="37" t="n"/>
+      <c r="K2" s="50" t="n"/>
       <c r="L2" s="38" t="n"/>
       <c r="M2" s="38" t="n"/>
       <c r="N2" s="38" t="n"/>
@@ -1211,17 +1259,17 @@
           <t>Модель изделия: XXX</t>
         </is>
       </c>
-      <c r="B3" s="40" t="n"/>
-      <c r="C3" s="40" t="n"/>
+      <c r="B3" s="51" t="n"/>
+      <c r="C3" s="51" t="n"/>
       <c r="D3" s="40" t="inlineStr">
         <is>
           <t>Версия:</t>
         </is>
       </c>
-      <c r="E3" s="40" t="n"/>
-      <c r="F3" s="40" t="n"/>
-      <c r="G3" s="40" t="n"/>
-      <c r="H3" s="40" t="n"/>
+      <c r="E3" s="51" t="n"/>
+      <c r="F3" s="51" t="n"/>
+      <c r="G3" s="51" t="n"/>
+      <c r="H3" s="51" t="n"/>
       <c r="I3" s="37" t="inlineStr">
         <is>
           <t>Проверил:</t>
@@ -1232,7 +1280,7 @@
           <t>Дата:</t>
         </is>
       </c>
-      <c r="K3" s="37" t="n"/>
+      <c r="K3" s="50" t="n"/>
       <c r="L3" s="38" t="n"/>
       <c r="M3" s="38" t="n"/>
       <c r="N3" s="38" t="n"/>
@@ -1261,7 +1309,7 @@
           <t>Дата:</t>
         </is>
       </c>
-      <c r="K4" s="37" t="n"/>
+      <c r="K4" s="50" t="n"/>
       <c r="L4" s="38" t="n"/>
       <c r="M4" s="38" t="n"/>
       <c r="N4" s="38" t="n"/>
@@ -1285,8 +1333,8 @@
           <t>Номер таблицы:</t>
         </is>
       </c>
-      <c r="J5" s="37" t="n"/>
-      <c r="K5" s="37" t="n"/>
+      <c r="J5" s="50" t="n"/>
+      <c r="K5" s="50" t="n"/>
       <c r="L5" s="38" t="n"/>
       <c r="M5" s="38" t="n"/>
       <c r="N5" s="38" t="n"/>
@@ -1346,7 +1394,7 @@
       </c>
       <c r="J6" s="41" t="inlineStr">
         <is>
-          <t>Масса ед. кг</t>
+          <t>Масса</t>
         </is>
       </c>
       <c r="K6" s="41" t="inlineStr">
@@ -1376,7 +1424,7 @@
       </c>
       <c r="P6" s="41" t="inlineStr">
         <is>
-          <t>Габаритные размеры</t>
+          <t>Габарит</t>
         </is>
       </c>
       <c r="Q6" s="35" t="n"/>
@@ -2752,14 +2800,14 @@
       <c r="A72" s="42" t="n"/>
       <c r="B72" s="43" t="n"/>
       <c r="C72" s="43" t="n"/>
-      <c r="D72" s="43" t="n"/>
-      <c r="E72" s="43" t="n"/>
+      <c r="D72" s="52" t="n"/>
+      <c r="E72" s="53" t="n"/>
       <c r="F72" s="43" t="n"/>
-      <c r="G72" s="42" t="n"/>
+      <c r="G72" s="53" t="n"/>
       <c r="H72" s="43" t="n"/>
-      <c r="I72" s="43" t="n"/>
-      <c r="J72" s="42" t="n"/>
-      <c r="K72" s="43" t="n"/>
+      <c r="I72" s="52" t="n"/>
+      <c r="J72" s="52" t="n"/>
+      <c r="K72" s="53" t="n"/>
       <c r="L72" s="43" t="n"/>
       <c r="M72" s="43" t="n"/>
       <c r="N72" s="43" t="n"/>
@@ -2772,15 +2820,14 @@
     <row r="73" ht="20" customHeight="1">
       <c r="A73" s="42" t="n"/>
       <c r="B73" s="49" t="n"/>
-      <c r="C73" s="43" t="n"/>
-      <c r="D73" s="43" t="n"/>
-      <c r="E73" s="43" t="n"/>
-      <c r="F73" s="43" t="n"/>
-      <c r="G73" s="42" t="n"/>
-      <c r="H73" s="43" t="n"/>
-      <c r="I73" s="43" t="n"/>
-      <c r="J73" s="42" t="n"/>
-      <c r="K73" s="43" t="n"/>
+      <c r="C73" s="54" t="n"/>
+      <c r="E73" s="55" t="n"/>
+      <c r="F73" s="56" t="n"/>
+      <c r="G73" s="57" t="n"/>
+      <c r="H73" s="56" t="n"/>
+      <c r="I73" s="58" t="n"/>
+      <c r="J73" s="58" t="n"/>
+      <c r="K73" s="57" t="n"/>
       <c r="L73" s="43" t="n"/>
       <c r="M73" s="43" t="n"/>
       <c r="N73" s="43" t="n"/>
@@ -2793,15 +2840,14 @@
     <row r="74" ht="20" customHeight="1">
       <c r="A74" s="42" t="n"/>
       <c r="B74" s="43" t="n"/>
-      <c r="C74" s="43" t="n"/>
-      <c r="D74" s="43" t="n"/>
-      <c r="E74" s="43" t="n"/>
+      <c r="C74" s="54" t="n"/>
+      <c r="E74" s="55" t="n"/>
       <c r="F74" s="43" t="n"/>
-      <c r="G74" s="42" t="n"/>
+      <c r="G74" s="53" t="n"/>
       <c r="H74" s="43" t="n"/>
-      <c r="I74" s="43" t="n"/>
-      <c r="J74" s="42" t="n"/>
-      <c r="K74" s="43" t="n"/>
+      <c r="I74" s="52" t="n"/>
+      <c r="J74" s="52" t="n"/>
+      <c r="K74" s="53" t="n"/>
       <c r="L74" s="43" t="n"/>
       <c r="M74" s="43" t="n"/>
       <c r="N74" s="43" t="n"/>
@@ -2814,15 +2860,15 @@
     <row r="75" ht="20" customHeight="1">
       <c r="A75" s="42" t="n"/>
       <c r="B75" s="43" t="n"/>
-      <c r="C75" s="43" t="n"/>
-      <c r="D75" s="43" t="n"/>
-      <c r="E75" s="43" t="n"/>
-      <c r="F75" s="43" t="n"/>
-      <c r="G75" s="42" t="n"/>
-      <c r="H75" s="43" t="n"/>
-      <c r="I75" s="43" t="n"/>
-      <c r="J75" s="42" t="n"/>
-      <c r="K75" s="43" t="n"/>
+      <c r="C75" s="56" t="n"/>
+      <c r="D75" s="58" t="n"/>
+      <c r="E75" s="57" t="n"/>
+      <c r="F75" s="56" t="n"/>
+      <c r="G75" s="57" t="n"/>
+      <c r="H75" s="56" t="n"/>
+      <c r="I75" s="58" t="n"/>
+      <c r="J75" s="58" t="n"/>
+      <c r="K75" s="57" t="n"/>
       <c r="L75" s="43" t="n"/>
       <c r="M75" s="43" t="n"/>
       <c r="N75" s="43" t="n"/>

</xml_diff>

<commit_message>
fix: align calculated BOM anchors
</commit_message>
<xml_diff>
--- a/Шаблоны спецификации/bom_шаблон.xlsx
+++ b/Шаблоны спецификации/bom_шаблон.xlsx
@@ -17,12 +17,12 @@
     <definedName name="Количество">'Спецификация'!$G$6</definedName>
     <definedName name="Тип">'Спецификация'!$H$6</definedName>
     <definedName name="ОбработкаПоверхности">'Спецификация'!$I$6</definedName>
-    <definedName name="МассаЕдКг">'Спецификация'!$J$6</definedName>
     <definedName name="ИмяФайла">'Спецификация'!$L$6</definedName>
     <definedName name="Эскиз">'Спецификация'!$M$6</definedName>
     <definedName name="Материал">'Спецификация'!$N$6</definedName>
     <definedName name="Путь">'Спецификация'!$O$6</definedName>
-    <definedName name="ГабаритныеРазмеры">'Спецификация'!$P$6</definedName>
+    <definedName name="Масса">'Спецификация'!$J$6</definedName>
+    <definedName name="Габарит">'Спецификация'!$P$6</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Спецификация'!$1:$6</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'Спецификация'!$A$1:$P$75</definedName>
   </definedNames>

</xml_diff>